<commit_message>
mer jobb på excelfilen
</commit_message>
<xml_diff>
--- a/ET2/Radialpump-lab_Grupp-5.xlsx
+++ b/ET2/Radialpump-lab_Grupp-5.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{469FFC67-6F24-4F7F-9BBB-363A1D81C9A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A67974D4-34C1-4148-8FFD-0BBA77E444AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="34605" windowHeight="21705" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,6 @@
     <definedName name="π">Sheet1!$B$10</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -56,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="233" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="118">
   <si>
     <t>Pin</t>
   </si>
@@ -532,15 +531,22 @@
   <si>
     <t>Grupp 5: Emil Persson, Johan Hammar</t>
   </si>
+  <si>
+    <t>alt ekvation(Swamee &amp; Jain)</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
+  <numFmts count="7">
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
+    <numFmt numFmtId="175" formatCode="0.0000"/>
+    <numFmt numFmtId="176" formatCode="0.00000"/>
+    <numFmt numFmtId="178" formatCode="0.0000000"/>
+    <numFmt numFmtId="179" formatCode="0.00000000"/>
   </numFmts>
   <fonts count="19" x14ac:knownFonts="1">
     <font>
@@ -688,12 +694,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFC000"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="8" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -701,6 +701,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0" tint="-4.9989318521683403E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -742,7 +748,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -817,9 +823,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="2" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -834,10 +837,10 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="165" fontId="18" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="18" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="3" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -846,10 +849,10 @@
     <xf numFmtId="9" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="10" fontId="3" fillId="6" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="10" fontId="3" fillId="5" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="2" fontId="3" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -868,6 +871,21 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="166" fontId="3" fillId="3" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="175" fontId="3" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="3" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="3" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="3" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -991,7 +1009,19 @@
             <a:effectLst/>
           </c:spPr>
           <c:marker>
-            <c:symbol val="none"/>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
           </c:marker>
           <c:xVal>
             <c:numRef>
@@ -1094,7 +1124,19 @@
             <a:effectLst/>
           </c:spPr>
           <c:marker>
-            <c:symbol val="none"/>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent2"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
           </c:marker>
           <c:xVal>
             <c:numRef>
@@ -1455,8 +1497,8 @@
           <c:yMode val="edge"/>
           <c:x val="0.87572437511143886"/>
           <c:y val="0.10404488586199889"/>
-          <c:w val="0.10890210974415881"/>
-          <c:h val="8.1476285790863329E-2"/>
+          <c:w val="0.10908942435508184"/>
+          <c:h val="8.0431200163028627E-2"/>
         </c:manualLayout>
       </c:layout>
       <c:overlay val="0"/>
@@ -3170,8 +3212,8 @@
           <c:yMode val="edge"/>
           <c:x val="0.71274053861789655"/>
           <c:y val="0.10811445399916456"/>
-          <c:w val="0.28725952937103788"/>
-          <c:h val="0.60966925389349025"/>
+          <c:w val="0.28725953312603214"/>
+          <c:h val="0.60107588982202598"/>
         </c:manualLayout>
       </c:layout>
       <c:overlay val="0"/>
@@ -6822,16 +6864,16 @@
       <c r="F5" s="10" t="s">
         <v>92</v>
       </c>
-      <c r="G5" s="54">
+      <c r="G5" s="53">
         <v>179</v>
       </c>
-      <c r="H5" s="54">
+      <c r="H5" s="53">
         <v>136</v>
       </c>
-      <c r="I5" s="54">
+      <c r="I5" s="53">
         <v>60.9</v>
       </c>
-      <c r="J5" s="55">
+      <c r="J5" s="54">
         <v>39.22</v>
       </c>
       <c r="U5" s="5"/>
@@ -6840,16 +6882,16 @@
       <c r="A6" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="G6" s="54">
+      <c r="G6" s="53">
         <v>179</v>
       </c>
-      <c r="H6" s="54">
+      <c r="H6" s="53">
         <v>142</v>
       </c>
-      <c r="I6" s="54">
+      <c r="I6" s="53">
         <v>61.1</v>
       </c>
-      <c r="J6" s="55">
+      <c r="J6" s="54">
         <v>39.119999999999997</v>
       </c>
       <c r="U6" s="5"/>
@@ -6864,16 +6906,16 @@
       <c r="C7" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="G7" s="54">
+      <c r="G7" s="53">
         <v>180</v>
       </c>
-      <c r="H7" s="54">
+      <c r="H7" s="53">
         <v>135</v>
       </c>
-      <c r="I7" s="54">
+      <c r="I7" s="53">
         <v>60.9</v>
       </c>
-      <c r="J7" s="55">
+      <c r="J7" s="54">
         <v>38.96</v>
       </c>
     </row>
@@ -6887,16 +6929,16 @@
       <c r="C8" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="G8" s="54">
+      <c r="G8" s="53">
         <v>179.5</v>
       </c>
-      <c r="H8" s="54">
+      <c r="H8" s="53">
         <v>136.5</v>
       </c>
-      <c r="I8" s="54">
+      <c r="I8" s="53">
         <v>61.09</v>
       </c>
-      <c r="J8" s="55">
+      <c r="J8" s="54">
         <v>39.1</v>
       </c>
     </row>
@@ -6911,16 +6953,16 @@
         <v>62</v>
       </c>
       <c r="F9" s="12"/>
-      <c r="G9" s="54">
+      <c r="G9" s="53">
         <v>179.5</v>
       </c>
-      <c r="H9" s="54">
+      <c r="H9" s="53">
         <v>137</v>
       </c>
-      <c r="I9" s="54">
+      <c r="I9" s="53">
         <v>60.8</v>
       </c>
-      <c r="J9" s="55">
+      <c r="J9" s="54">
         <v>39.26</v>
       </c>
     </row>
@@ -6933,16 +6975,16 @@
         <v>3.1415926535897931</v>
       </c>
       <c r="F10" s="12"/>
-      <c r="G10" s="54">
+      <c r="G10" s="53">
         <v>179</v>
       </c>
-      <c r="H10" s="54">
+      <c r="H10" s="53">
         <v>137</v>
       </c>
-      <c r="I10" s="54">
+      <c r="I10" s="53">
         <v>60.8</v>
       </c>
-      <c r="J10" s="55">
+      <c r="J10" s="54">
         <v>39.1</v>
       </c>
     </row>
@@ -7067,7 +7109,7 @@
       <c r="A17" s="11">
         <v>15600</v>
       </c>
-      <c r="B17" s="54">
+      <c r="B17" s="53">
         <v>-5</v>
       </c>
       <c r="C17" s="11">
@@ -7082,11 +7124,11 @@
       <c r="F17" s="11">
         <v>39.1</v>
       </c>
-      <c r="G17" s="51">
+      <c r="G17" s="50">
         <f>D17/3</f>
         <v>2219.3333333333335</v>
       </c>
-      <c r="H17" s="51">
+      <c r="H17" s="50">
         <f>G17/1.5</f>
         <v>1479.5555555555557</v>
       </c>
@@ -7094,27 +7136,27 @@
         <f>1-(G17/(30*2*F17))</f>
         <v>5.3992611537368451E-2</v>
       </c>
-      <c r="J17" s="52">
+      <c r="J17" s="51">
         <f>((E17/1000)*Tyngdacc)*Hävarm</f>
         <v>1.3440746400000003</v>
       </c>
-      <c r="K17" s="51">
+      <c r="K17" s="50">
         <f>A17/1000</f>
         <v>15.6</v>
       </c>
-      <c r="L17" s="52">
+      <c r="L17" s="51">
         <f t="shared" ref="L17:L26" si="0">delta_z+((C17-ABS(B17/10))*1000/(Densitet*Tyngdacc))+(((4*(K17/3600))/(π*PumpDiam_tryck^2))^2-((4*(K17/3600))/(π*PumpDiam_sug^2))^2)/(2*Tyngdacc)</f>
         <v>2.6780641029119727</v>
       </c>
-      <c r="M17" s="51">
+      <c r="M17" s="50">
         <f t="shared" ref="M17:M26" si="1">Densitet*Tyngdacc*(K17/3600)*L17</f>
         <v>113.63958490576134</v>
       </c>
-      <c r="N17" s="51">
+      <c r="N17" s="50">
         <f t="shared" ref="N17:N26" si="2">((G17*2*π)/60)*J17</f>
         <v>312.37375699118348</v>
       </c>
-      <c r="O17" s="56">
+      <c r="O17" s="55">
         <f>M17/N17</f>
         <v>0.36379363618874272</v>
       </c>
@@ -7123,7 +7165,7 @@
       <c r="A18" s="11">
         <v>14000</v>
       </c>
-      <c r="B18" s="54">
+      <c r="B18" s="53">
         <v>2.5</v>
       </c>
       <c r="C18" s="11">
@@ -7138,11 +7180,11 @@
       <c r="F18" s="11">
         <v>39.1</v>
       </c>
-      <c r="G18" s="51">
+      <c r="G18" s="50">
         <f t="shared" ref="G18:G26" si="3">D18/3</f>
         <v>2221.6666666666665</v>
       </c>
-      <c r="H18" s="51">
+      <c r="H18" s="50">
         <f t="shared" ref="H18:H26" si="4">G18/1.5</f>
         <v>1481.1111111111111</v>
       </c>
@@ -7150,27 +7192,27 @@
         <f t="shared" ref="I18:I26" si="5">1-(G18/(30*2*F18))</f>
         <v>5.2998010798522399E-2</v>
       </c>
-      <c r="J18" s="52">
+      <c r="J18" s="51">
         <f t="shared" ref="J18:J26" si="6">((E18/1000)*Tyngdacc)*Hävarm</f>
         <v>1.3423153800000001</v>
       </c>
-      <c r="K18" s="51">
+      <c r="K18" s="50">
         <f t="shared" ref="K18:K26" si="7">A18/1000</f>
         <v>14</v>
       </c>
-      <c r="L18" s="52">
+      <c r="L18" s="51">
         <f t="shared" si="0"/>
         <v>3.6178702573899622</v>
       </c>
-      <c r="M18" s="51">
+      <c r="M18" s="50">
         <f t="shared" si="1"/>
         <v>137.7733111688521</v>
       </c>
-      <c r="N18" s="51">
+      <c r="N18" s="50">
         <f t="shared" si="2"/>
         <v>312.29288033884734</v>
       </c>
-      <c r="O18" s="56">
+      <c r="O18" s="55">
         <f t="shared" ref="O18:O26" si="8">M18/N18</f>
         <v>0.44116699368670792</v>
       </c>
@@ -7179,7 +7221,7 @@
       <c r="A19" s="11">
         <v>13000</v>
       </c>
-      <c r="B19" s="54">
+      <c r="B19" s="53">
         <v>6.5</v>
       </c>
       <c r="C19" s="11">
@@ -7194,11 +7236,11 @@
       <c r="F19" s="11">
         <v>39.1</v>
       </c>
-      <c r="G19" s="51">
+      <c r="G19" s="50">
         <f>D19/3</f>
         <v>2224.3333333333335</v>
       </c>
-      <c r="H19" s="51">
+      <c r="H19" s="50">
         <f t="shared" si="4"/>
         <v>1482.8888888888889</v>
       </c>
@@ -7206,27 +7248,27 @@
         <f t="shared" si="5"/>
         <v>5.18613242398408E-2</v>
       </c>
-      <c r="J19" s="52">
+      <c r="J19" s="51">
         <f t="shared" si="6"/>
         <v>1.3229635200000003</v>
       </c>
-      <c r="K19" s="51">
+      <c r="K19" s="50">
         <f t="shared" si="7"/>
         <v>13</v>
       </c>
-      <c r="L19" s="52">
+      <c r="L19" s="51">
         <f t="shared" si="0"/>
         <v>4.0266640621808545</v>
       </c>
-      <c r="M19" s="51">
+      <c r="M19" s="50">
         <f t="shared" si="1"/>
         <v>142.38781416883182</v>
       </c>
-      <c r="N19" s="51">
+      <c r="N19" s="50">
         <f t="shared" si="2"/>
         <v>308.16006498154991</v>
       </c>
-      <c r="O19" s="56">
+      <c r="O19" s="55">
         <f t="shared" si="8"/>
         <v>0.46205797035172885</v>
       </c>
@@ -7235,7 +7277,7 @@
       <c r="A20" s="11">
         <v>11800</v>
       </c>
-      <c r="B20" s="54">
+      <c r="B20" s="53">
         <v>12</v>
       </c>
       <c r="C20" s="11">
@@ -7250,11 +7292,11 @@
       <c r="F20" s="11">
         <v>39.1</v>
       </c>
-      <c r="G20" s="51">
+      <c r="G20" s="50">
         <f t="shared" si="3"/>
         <v>2225</v>
       </c>
-      <c r="H20" s="51">
+      <c r="H20" s="50">
         <f t="shared" si="4"/>
         <v>1483.3333333333333</v>
       </c>
@@ -7262,27 +7304,27 @@
         <f t="shared" si="5"/>
         <v>5.1577152600170484E-2</v>
       </c>
-      <c r="J20" s="52">
+      <c r="J20" s="51">
         <f t="shared" si="6"/>
         <v>1.3018524000000002</v>
       </c>
-      <c r="K20" s="51">
+      <c r="K20" s="50">
         <f t="shared" si="7"/>
         <v>11.8</v>
       </c>
-      <c r="L20" s="52">
+      <c r="L20" s="51">
         <f t="shared" si="0"/>
         <v>4.4139082025556826</v>
       </c>
-      <c r="M20" s="51">
+      <c r="M20" s="50">
         <f t="shared" si="1"/>
         <v>141.67374566032225</v>
       </c>
-      <c r="N20" s="51">
+      <c r="N20" s="50">
         <f t="shared" si="2"/>
         <v>303.33350357911957</v>
       </c>
-      <c r="O20" s="56">
+      <c r="O20" s="55">
         <f t="shared" si="8"/>
         <v>0.46705604223955755</v>
       </c>
@@ -7291,7 +7333,7 @@
       <c r="A21" s="11">
         <v>9500</v>
       </c>
-      <c r="B21" s="54">
+      <c r="B21" s="53">
         <v>20</v>
       </c>
       <c r="C21" s="11">
@@ -7306,11 +7348,11 @@
       <c r="F21" s="11">
         <v>39.200000000000003</v>
       </c>
-      <c r="G21" s="51">
+      <c r="G21" s="50">
         <f t="shared" si="3"/>
         <v>2232.6666666666665</v>
       </c>
-      <c r="H21" s="51">
+      <c r="H21" s="50">
         <f t="shared" si="4"/>
         <v>1488.4444444444443</v>
       </c>
@@ -7318,27 +7360,27 @@
         <f t="shared" si="5"/>
         <v>5.0736961451247176E-2</v>
       </c>
-      <c r="J21" s="52">
+      <c r="J21" s="51">
         <f t="shared" si="6"/>
         <v>1.2279634800000001</v>
       </c>
-      <c r="K21" s="51">
+      <c r="K21" s="50">
         <f t="shared" si="7"/>
         <v>9.5</v>
       </c>
-      <c r="L21" s="52">
+      <c r="L21" s="51">
         <f t="shared" si="0"/>
         <v>5.1406868536623485</v>
       </c>
-      <c r="M21" s="51">
+      <c r="M21" s="50">
         <f t="shared" si="1"/>
         <v>132.83998776852053</v>
       </c>
-      <c r="N21" s="51">
+      <c r="N21" s="50">
         <f t="shared" si="2"/>
         <v>287.10314996803606</v>
       </c>
-      <c r="O21" s="56">
+      <c r="O21" s="55">
         <f t="shared" si="8"/>
         <v>0.46269080566796272</v>
       </c>
@@ -7347,7 +7389,7 @@
       <c r="A22" s="11">
         <v>8100</v>
       </c>
-      <c r="B22" s="54">
+      <c r="B22" s="53">
         <v>25</v>
       </c>
       <c r="C22" s="11">
@@ -7362,11 +7404,11 @@
       <c r="F22" s="11">
         <v>39.200000000000003</v>
       </c>
-      <c r="G22" s="51">
+      <c r="G22" s="50">
         <f t="shared" si="3"/>
         <v>2240.6666666666665</v>
       </c>
-      <c r="H22" s="51">
+      <c r="H22" s="50">
         <f t="shared" si="4"/>
         <v>1493.7777777777776</v>
       </c>
@@ -7374,27 +7416,27 @@
         <f t="shared" si="5"/>
         <v>4.7335600907029596E-2</v>
       </c>
-      <c r="J22" s="52">
+      <c r="J22" s="51">
         <f t="shared" si="6"/>
         <v>1.1663893800000003</v>
       </c>
-      <c r="K22" s="51">
+      <c r="K22" s="50">
         <f t="shared" si="7"/>
         <v>8.1</v>
       </c>
-      <c r="L22" s="52">
+      <c r="L22" s="51">
         <f t="shared" si="0"/>
         <v>5.5445970424230921</v>
       </c>
-      <c r="M22" s="51">
+      <c r="M22" s="50">
         <f t="shared" si="1"/>
         <v>122.16282860608972</v>
       </c>
-      <c r="N22" s="51">
+      <c r="N22" s="50">
         <f t="shared" si="2"/>
         <v>273.684012295174</v>
       </c>
-      <c r="O22" s="56">
+      <c r="O22" s="55">
         <f t="shared" si="8"/>
         <v>0.44636450474985923</v>
       </c>
@@ -7403,7 +7445,7 @@
       <c r="A23" s="11">
         <v>7200</v>
       </c>
-      <c r="B23" s="54">
+      <c r="B23" s="53">
         <v>27</v>
       </c>
       <c r="C23" s="11">
@@ -7418,11 +7460,11 @@
       <c r="F23" s="11">
         <v>39.200000000000003</v>
       </c>
-      <c r="G23" s="51">
+      <c r="G23" s="50">
         <f t="shared" si="3"/>
         <v>2244.6666666666665</v>
       </c>
-      <c r="H23" s="51">
+      <c r="H23" s="50">
         <f t="shared" si="4"/>
         <v>1496.4444444444443</v>
       </c>
@@ -7430,27 +7472,27 @@
         <f t="shared" si="5"/>
         <v>4.5634920634920695E-2</v>
       </c>
-      <c r="J23" s="52">
+      <c r="J23" s="51">
         <f t="shared" si="6"/>
         <v>1.1259264000000002</v>
       </c>
-      <c r="K23" s="51">
+      <c r="K23" s="50">
         <f t="shared" si="7"/>
         <v>7.2</v>
       </c>
-      <c r="L23" s="52">
+      <c r="L23" s="51">
         <f t="shared" si="0"/>
         <v>5.6973240263700138</v>
       </c>
-      <c r="M23" s="51">
+      <c r="M23" s="50">
         <f t="shared" si="1"/>
         <v>111.5802907020644</v>
       </c>
-      <c r="N23" s="51">
+      <c r="N23" s="50">
         <f t="shared" si="2"/>
         <v>264.66132207412619</v>
       </c>
-      <c r="O23" s="56">
+      <c r="O23" s="55">
         <f t="shared" si="8"/>
         <v>0.42159651371654927</v>
       </c>
@@ -7459,7 +7501,7 @@
       <c r="A24" s="11">
         <v>6400</v>
       </c>
-      <c r="B24" s="54">
+      <c r="B24" s="53">
         <v>30</v>
       </c>
       <c r="C24" s="11">
@@ -7474,11 +7516,11 @@
       <c r="F24" s="11">
         <v>39.200000000000003</v>
       </c>
-      <c r="G24" s="51">
+      <c r="G24" s="50">
         <f t="shared" si="3"/>
         <v>2248.6666666666665</v>
       </c>
-      <c r="H24" s="51">
+      <c r="H24" s="50">
         <f t="shared" si="4"/>
         <v>1499.1111111111111</v>
       </c>
@@ -7486,27 +7528,27 @@
         <f t="shared" si="5"/>
         <v>4.3934240362811905E-2</v>
       </c>
-      <c r="J24" s="52">
+      <c r="J24" s="51">
         <f t="shared" si="6"/>
         <v>1.0872226800000002</v>
       </c>
-      <c r="K24" s="51">
+      <c r="K24" s="50">
         <f t="shared" si="7"/>
         <v>6.4</v>
       </c>
-      <c r="L24" s="52">
+      <c r="L24" s="51">
         <f t="shared" si="0"/>
         <v>5.8463640367306828</v>
       </c>
-      <c r="M24" s="51">
+      <c r="M24" s="50">
         <f t="shared" si="1"/>
         <v>101.77705974074206</v>
       </c>
-      <c r="N24" s="51">
+      <c r="N24" s="50">
         <f t="shared" si="2"/>
         <v>256.01900389906865</v>
       </c>
-      <c r="O24" s="56">
+      <c r="O24" s="55">
         <f t="shared" si="8"/>
         <v>0.39753712884870851</v>
       </c>
@@ -7515,7 +7557,7 @@
       <c r="A25" s="11">
         <v>5500</v>
       </c>
-      <c r="B25" s="54">
+      <c r="B25" s="53">
         <v>34</v>
       </c>
       <c r="C25" s="11">
@@ -7530,11 +7572,11 @@
       <c r="F25" s="11">
         <v>39.200000000000003</v>
       </c>
-      <c r="G25" s="51">
+      <c r="G25" s="50">
         <f t="shared" si="3"/>
         <v>2254.6666666666665</v>
       </c>
-      <c r="H25" s="51">
+      <c r="H25" s="50">
         <f t="shared" si="4"/>
         <v>1503.1111111111111</v>
       </c>
@@ -7542,27 +7584,27 @@
         <f t="shared" si="5"/>
         <v>4.1383219954648554E-2</v>
       </c>
-      <c r="J25" s="52">
+      <c r="J25" s="51">
         <f t="shared" si="6"/>
         <v>1.0379634</v>
       </c>
-      <c r="K25" s="51">
+      <c r="K25" s="50">
         <f t="shared" si="7"/>
         <v>5.5</v>
       </c>
-      <c r="L25" s="52">
+      <c r="L25" s="51">
         <f t="shared" si="0"/>
         <v>5.9855758141703879</v>
       </c>
-      <c r="M25" s="51">
+      <c r="M25" s="50">
         <f t="shared" si="1"/>
         <v>89.547341643351913</v>
       </c>
-      <c r="N25" s="51">
+      <c r="N25" s="50">
         <f t="shared" si="2"/>
         <v>245.07160901779673</v>
       </c>
-      <c r="O25" s="56">
+      <c r="O25" s="55">
         <f t="shared" si="8"/>
         <v>0.36539255608693993</v>
       </c>
@@ -7571,7 +7613,7 @@
       <c r="A26" s="11">
         <v>4800</v>
       </c>
-      <c r="B26" s="54">
+      <c r="B26" s="53">
         <v>38</v>
       </c>
       <c r="C26" s="11">
@@ -7586,11 +7628,11 @@
       <c r="F26" s="11">
         <v>39.200000000000003</v>
       </c>
-      <c r="G26" s="51">
+      <c r="G26" s="50">
         <f t="shared" si="3"/>
         <v>2261.3333333333335</v>
       </c>
-      <c r="H26" s="51">
+      <c r="H26" s="50">
         <f t="shared" si="4"/>
         <v>1507.5555555555557</v>
       </c>
@@ -7598,27 +7640,27 @@
         <f t="shared" si="5"/>
         <v>3.8548752834467015E-2</v>
       </c>
-      <c r="J26" s="52">
+      <c r="J26" s="51">
         <f t="shared" si="6"/>
         <v>0.98518560000000022</v>
       </c>
-      <c r="K26" s="51">
+      <c r="K26" s="50">
         <f t="shared" si="7"/>
         <v>4.8</v>
       </c>
-      <c r="L26" s="52">
+      <c r="L26" s="51">
         <f t="shared" si="0"/>
         <v>6.0305693310778379</v>
       </c>
-      <c r="M26" s="51">
+      <c r="M26" s="50">
         <f t="shared" si="1"/>
         <v>78.737863126167227</v>
       </c>
-      <c r="N26" s="51">
+      <c r="N26" s="50">
         <f t="shared" si="2"/>
         <v>233.29813006118403</v>
       </c>
-      <c r="O26" s="56">
+      <c r="O26" s="55">
         <f t="shared" si="8"/>
         <v>0.33749890367967239</v>
       </c>
@@ -7754,7 +7796,7 @@
       <c r="A32" s="11">
         <v>12400</v>
       </c>
-      <c r="B32" s="54">
+      <c r="B32" s="53">
         <v>9</v>
       </c>
       <c r="C32" s="11">
@@ -7769,11 +7811,11 @@
       <c r="F32" s="11">
         <v>31.3</v>
       </c>
-      <c r="G32" s="51">
+      <c r="G32" s="50">
         <f>D32/3</f>
         <v>1780.6666666666667</v>
       </c>
-      <c r="H32" s="51">
+      <c r="H32" s="50">
         <f>G32/1.5</f>
         <v>1187.1111111111111</v>
       </c>
@@ -7781,27 +7823,27 @@
         <f>1-(G32/(30*2*F32))</f>
         <v>5.1828186013489486E-2</v>
       </c>
-      <c r="J32" s="52">
+      <c r="J32" s="51">
         <f t="shared" ref="J32:J41" si="9">((E32/1000)*Tyngdacc)*Hävarm</f>
         <v>0.98518560000000022</v>
       </c>
-      <c r="K32" s="51">
+      <c r="K32" s="50">
         <f>A32/1000</f>
         <v>12.4</v>
       </c>
-      <c r="L32" s="52">
+      <c r="L32" s="51">
         <f t="shared" ref="L32:L41" si="10">delta_z+((C32-ABS(B32/10))*1000/(Densitet*Tyngdacc))+(((4*(K32/3600))/(π*PumpDiam_tryck^2))^2-((4*(K32/3600))/(π*PumpDiam_sug^2))^2)/(2*Tyngdacc)</f>
         <v>1.9243124674288614</v>
       </c>
-      <c r="M32" s="51">
+      <c r="M32" s="50">
         <f t="shared" ref="M32:M41" si="11">Densitet*Tyngdacc*(K32/3600)*L32</f>
         <v>64.905477741527278</v>
       </c>
-      <c r="N32" s="51">
+      <c r="N32" s="50">
         <f t="shared" ref="N32:N41" si="12">((G32*2*π)/60)*J32</f>
         <v>183.70852163721185</v>
       </c>
-      <c r="O32" s="56">
+      <c r="O32" s="55">
         <f>M32/N32</f>
         <v>0.35330684261725659</v>
       </c>
@@ -7813,7 +7855,7 @@
       <c r="A33" s="11">
         <v>11400</v>
       </c>
-      <c r="B33" s="54">
+      <c r="B33" s="53">
         <v>13</v>
       </c>
       <c r="C33" s="11">
@@ -7828,11 +7870,11 @@
       <c r="F33" s="11">
         <v>31.3</v>
       </c>
-      <c r="G33" s="51">
+      <c r="G33" s="50">
         <f t="shared" ref="G33:G41" si="13">D33/3</f>
         <v>1782.6666666666667</v>
       </c>
-      <c r="H33" s="51">
+      <c r="H33" s="50">
         <f t="shared" ref="H33:H41" si="14">G33/1.5</f>
         <v>1188.4444444444446</v>
       </c>
@@ -7840,27 +7882,27 @@
         <f t="shared" ref="I33:I41" si="15">1-(G33/(30*2*F33))</f>
         <v>5.0763223287184855E-2</v>
       </c>
-      <c r="J33" s="52">
+      <c r="J33" s="51">
         <f t="shared" si="9"/>
         <v>0.97638930000000013</v>
       </c>
-      <c r="K33" s="51">
+      <c r="K33" s="50">
         <f t="shared" ref="K33:K41" si="16">A33/1000</f>
         <v>11.4</v>
       </c>
-      <c r="L33" s="52">
+      <c r="L33" s="51">
         <f t="shared" si="10"/>
         <v>2.2382106669079334</v>
       </c>
-      <c r="M33" s="51">
+      <c r="M33" s="50">
         <f t="shared" si="11"/>
         <v>69.404860341633466</v>
       </c>
-      <c r="N33" s="51">
+      <c r="N33" s="50">
         <f t="shared" si="12"/>
         <v>182.2727614765316</v>
       </c>
-      <c r="O33" s="56">
+      <c r="O33" s="55">
         <f t="shared" ref="O33:O41" si="17">M33/N33</f>
         <v>0.38077472343869462</v>
       </c>
@@ -7872,7 +7914,7 @@
       <c r="A34" s="11">
         <v>10500</v>
       </c>
-      <c r="B34" s="54">
+      <c r="B34" s="53">
         <v>16</v>
       </c>
       <c r="C34" s="11">
@@ -7887,11 +7929,11 @@
       <c r="F34" s="11">
         <v>31.3</v>
       </c>
-      <c r="G34" s="51">
+      <c r="G34" s="50">
         <f t="shared" si="13"/>
         <v>1784</v>
       </c>
-      <c r="H34" s="51">
+      <c r="H34" s="50">
         <f t="shared" si="14"/>
         <v>1189.3333333333333</v>
       </c>
@@ -7899,27 +7941,27 @@
         <f t="shared" si="15"/>
         <v>5.0053248136315176E-2</v>
       </c>
-      <c r="J34" s="52">
+      <c r="J34" s="51">
         <f t="shared" si="9"/>
         <v>0.95879670000000017</v>
       </c>
-      <c r="K34" s="51">
+      <c r="K34" s="50">
         <f t="shared" si="16"/>
         <v>10.5</v>
       </c>
-      <c r="L34" s="52">
+      <c r="L34" s="51">
         <f t="shared" si="10"/>
         <v>2.5715553951777754</v>
       </c>
-      <c r="M34" s="51">
+      <c r="M34" s="50">
         <f t="shared" si="11"/>
         <v>73.446187212783968</v>
       </c>
-      <c r="N34" s="51">
+      <c r="N34" s="50">
         <f t="shared" si="12"/>
         <v>179.12244085023164</v>
       </c>
-      <c r="O34" s="56">
+      <c r="O34" s="55">
         <f t="shared" si="17"/>
         <v>0.41003342107309715</v>
       </c>
@@ -7931,7 +7973,7 @@
       <c r="A35" s="11">
         <v>9600</v>
       </c>
-      <c r="B35" s="54">
+      <c r="B35" s="53">
         <v>20</v>
       </c>
       <c r="C35" s="11">
@@ -7946,11 +7988,11 @@
       <c r="F35" s="11">
         <v>31.3</v>
       </c>
-      <c r="G35" s="51">
+      <c r="G35" s="50">
         <f t="shared" si="13"/>
         <v>1791.6666666666667</v>
       </c>
-      <c r="H35" s="51">
+      <c r="H35" s="50">
         <f t="shared" si="14"/>
         <v>1194.4444444444446</v>
       </c>
@@ -7958,27 +8000,27 @@
         <f t="shared" si="15"/>
         <v>4.5970891018814353E-2</v>
       </c>
-      <c r="J35" s="52">
+      <c r="J35" s="51">
         <f t="shared" si="9"/>
         <v>0.93768558000000013</v>
       </c>
-      <c r="K35" s="51">
+      <c r="K35" s="50">
         <f t="shared" si="16"/>
         <v>9.6</v>
       </c>
-      <c r="L35" s="52">
+      <c r="L35" s="51">
         <f t="shared" si="10"/>
         <v>2.8983457236278789</v>
       </c>
-      <c r="M35" s="51">
+      <c r="M35" s="50">
         <f t="shared" si="11"/>
         <v>75.684246826671128</v>
       </c>
-      <c r="N35" s="51">
+      <c r="N35" s="50">
         <f t="shared" si="12"/>
         <v>175.93128273433146</v>
       </c>
-      <c r="O35" s="56">
+      <c r="O35" s="55">
         <f t="shared" si="17"/>
         <v>0.4301920934718565</v>
       </c>
@@ -7990,7 +8032,7 @@
       <c r="A36" s="11">
         <v>8700</v>
       </c>
-      <c r="B36" s="54">
+      <c r="B36" s="53">
         <v>23</v>
       </c>
       <c r="C36" s="11">
@@ -8005,11 +8047,11 @@
       <c r="F36" s="11">
         <v>31.3</v>
       </c>
-      <c r="G36" s="51">
+      <c r="G36" s="50">
         <f t="shared" si="13"/>
         <v>1789.6666666666667</v>
       </c>
-      <c r="H36" s="51">
+      <c r="H36" s="50">
         <f t="shared" si="14"/>
         <v>1193.1111111111111</v>
       </c>
@@ -8017,27 +8059,27 @@
         <f t="shared" si="15"/>
         <v>4.7035853745118872E-2</v>
       </c>
-      <c r="J36" s="52">
+      <c r="J36" s="51">
         <f t="shared" si="9"/>
         <v>0.92361150000000014</v>
       </c>
-      <c r="K36" s="51">
+      <c r="K36" s="50">
         <f t="shared" si="16"/>
         <v>8.6999999999999993</v>
       </c>
-      <c r="L36" s="52">
+      <c r="L36" s="51">
         <f t="shared" si="10"/>
         <v>3.1368851592231763</v>
       </c>
-      <c r="M36" s="51">
+      <c r="M36" s="50">
         <f t="shared" si="11"/>
         <v>74.233843043441325</v>
       </c>
-      <c r="N36" s="51">
+      <c r="N36" s="50">
         <f t="shared" si="12"/>
         <v>173.09722236583741</v>
       </c>
-      <c r="O36" s="56">
+      <c r="O36" s="55">
         <f t="shared" si="17"/>
         <v>0.42885635037256475</v>
       </c>
@@ -8049,7 +8091,7 @@
       <c r="A37" s="11">
         <v>7900</v>
       </c>
-      <c r="B37" s="54">
+      <c r="B37" s="53">
         <v>25</v>
       </c>
       <c r="C37" s="11">
@@ -8064,11 +8106,11 @@
       <c r="F37" s="11">
         <v>31.3</v>
       </c>
-      <c r="G37" s="51">
+      <c r="G37" s="50">
         <f t="shared" si="13"/>
         <v>1791</v>
       </c>
-      <c r="H37" s="51">
+      <c r="H37" s="50">
         <f t="shared" si="14"/>
         <v>1194</v>
       </c>
@@ -8076,27 +8118,27 @@
         <f t="shared" si="15"/>
         <v>4.6325878594249192E-2</v>
       </c>
-      <c r="J37" s="52">
+      <c r="J37" s="51">
         <f t="shared" si="9"/>
         <v>0.8972226000000002</v>
       </c>
-      <c r="K37" s="51">
+      <c r="K37" s="50">
         <f t="shared" si="16"/>
         <v>7.9</v>
       </c>
-      <c r="L37" s="52">
+      <c r="L37" s="51">
         <f t="shared" si="10"/>
         <v>3.2907184729767183</v>
       </c>
-      <c r="M37" s="51">
+      <c r="M37" s="50">
         <f t="shared" si="11"/>
         <v>70.713428231537691</v>
       </c>
-      <c r="N37" s="51">
+      <c r="N37" s="50">
         <f t="shared" si="12"/>
         <v>168.27686334904561</v>
       </c>
-      <c r="O37" s="56">
+      <c r="O37" s="55">
         <f t="shared" si="17"/>
         <v>0.42022074112982177</v>
       </c>
@@ -8108,7 +8150,7 @@
       <c r="A38" s="11">
         <v>7000</v>
       </c>
-      <c r="B38" s="54">
+      <c r="B38" s="53">
         <v>27</v>
       </c>
       <c r="C38" s="11">
@@ -8123,11 +8165,11 @@
       <c r="F38" s="11">
         <v>31.3</v>
       </c>
-      <c r="G38" s="51">
+      <c r="G38" s="50">
         <f t="shared" si="13"/>
         <v>1794.6666666666667</v>
       </c>
-      <c r="H38" s="51">
+      <c r="H38" s="50">
         <f t="shared" si="14"/>
         <v>1196.4444444444446</v>
       </c>
@@ -8135,27 +8177,27 @@
         <f t="shared" si="15"/>
         <v>4.4373446929357407E-2</v>
       </c>
-      <c r="J38" s="52">
+      <c r="J38" s="51">
         <f t="shared" si="9"/>
         <v>0.87963000000000013</v>
       </c>
-      <c r="K38" s="51">
+      <c r="K38" s="50">
         <f t="shared" si="16"/>
         <v>7</v>
       </c>
-      <c r="L38" s="52">
+      <c r="L38" s="51">
         <f t="shared" si="10"/>
         <v>3.4442582706591165</v>
       </c>
-      <c r="M38" s="51">
+      <c r="M38" s="50">
         <f t="shared" si="11"/>
         <v>65.58096790509957</v>
       </c>
-      <c r="N38" s="51">
+      <c r="N38" s="50">
         <f t="shared" si="12"/>
         <v>165.31507068225326</v>
       </c>
-      <c r="O38" s="56">
+      <c r="O38" s="55">
         <f t="shared" si="17"/>
         <v>0.39670289970810113</v>
       </c>
@@ -8167,7 +8209,7 @@
       <c r="A39" s="11">
         <v>6200</v>
       </c>
-      <c r="B39" s="54">
+      <c r="B39" s="53">
         <v>29</v>
       </c>
       <c r="C39" s="11">
@@ -8182,11 +8224,11 @@
       <c r="F39" s="11">
         <v>31.3</v>
       </c>
-      <c r="G39" s="51">
+      <c r="G39" s="50">
         <f t="shared" si="13"/>
         <v>1798</v>
       </c>
-      <c r="H39" s="51">
+      <c r="H39" s="50">
         <f t="shared" si="14"/>
         <v>1198.6666666666667</v>
       </c>
@@ -8194,27 +8236,27 @@
         <f t="shared" si="15"/>
         <v>4.2598509052183209E-2</v>
       </c>
-      <c r="J39" s="52">
+      <c r="J39" s="51">
         <f t="shared" si="9"/>
         <v>0.84972258000000001</v>
       </c>
-      <c r="K39" s="51">
+      <c r="K39" s="50">
         <f t="shared" si="16"/>
         <v>6.2</v>
       </c>
-      <c r="L39" s="52">
+      <c r="L39" s="51">
         <f t="shared" si="10"/>
         <v>3.6042328437473707</v>
       </c>
-      <c r="M39" s="51">
+      <c r="M39" s="50">
         <f t="shared" si="11"/>
         <v>60.783905570100636</v>
       </c>
-      <c r="N39" s="51">
+      <c r="N39" s="50">
         <f t="shared" si="12"/>
         <v>159.99096741404745</v>
       </c>
-      <c r="O39" s="56">
+      <c r="O39" s="55">
         <f t="shared" si="17"/>
         <v>0.37992085773689571</v>
       </c>
@@ -8223,7 +8265,7 @@
       <c r="A40" s="11">
         <v>5400</v>
       </c>
-      <c r="B40" s="54">
+      <c r="B40" s="53">
         <v>31</v>
       </c>
       <c r="C40" s="11">
@@ -8238,11 +8280,11 @@
       <c r="F40" s="11">
         <v>31.4</v>
       </c>
-      <c r="G40" s="51">
+      <c r="G40" s="50">
         <f t="shared" si="13"/>
         <v>1801.3333333333333</v>
       </c>
-      <c r="H40" s="51">
+      <c r="H40" s="50">
         <f t="shared" si="14"/>
         <v>1200.8888888888889</v>
       </c>
@@ -8250,27 +8292,27 @@
         <f t="shared" si="15"/>
         <v>4.3878273177636262E-2</v>
       </c>
-      <c r="J40" s="52">
+      <c r="J40" s="51">
         <f t="shared" si="9"/>
         <v>0.81101886000000023</v>
       </c>
-      <c r="K40" s="51">
+      <c r="K40" s="50">
         <f t="shared" si="16"/>
         <v>5.4</v>
       </c>
-      <c r="L40" s="52">
+      <c r="L40" s="51">
         <f t="shared" si="10"/>
         <v>3.6649768049345961</v>
       </c>
-      <c r="M40" s="51">
+      <c r="M40" s="50">
         <f t="shared" si="11"/>
         <v>53.833059443980282</v>
       </c>
-      <c r="N40" s="51">
+      <c r="N40" s="50">
         <f t="shared" si="12"/>
         <v>152.98669314514834</v>
       </c>
-      <c r="O40" s="56">
+      <c r="O40" s="55">
         <f t="shared" si="17"/>
         <v>0.35188066580996941</v>
       </c>
@@ -8279,7 +8321,7 @@
       <c r="A41" s="11">
         <v>4400</v>
       </c>
-      <c r="B41" s="54">
+      <c r="B41" s="53">
         <v>35</v>
       </c>
       <c r="C41" s="11">
@@ -8294,11 +8336,11 @@
       <c r="F41" s="11">
         <v>31.4</v>
       </c>
-      <c r="G41" s="51">
+      <c r="G41" s="50">
         <f t="shared" si="13"/>
         <v>1806</v>
       </c>
-      <c r="H41" s="51">
+      <c r="H41" s="50">
         <f t="shared" si="14"/>
         <v>1204</v>
       </c>
@@ -8306,27 +8348,27 @@
         <f t="shared" si="15"/>
         <v>4.1401273885350309E-2</v>
       </c>
-      <c r="J41" s="52">
+      <c r="J41" s="51">
         <f t="shared" si="9"/>
         <v>0.77407440000000016</v>
       </c>
-      <c r="K41" s="51">
+      <c r="K41" s="50">
         <f t="shared" si="16"/>
         <v>4.4000000000000004</v>
       </c>
-      <c r="L41" s="52">
+      <c r="L41" s="51">
         <f t="shared" si="10"/>
         <v>3.8062431948723123</v>
       </c>
-      <c r="M41" s="51">
+      <c r="M41" s="50">
         <f t="shared" si="11"/>
         <v>45.5547095658873</v>
       </c>
-      <c r="N41" s="51">
+      <c r="N41" s="50">
         <f t="shared" si="12"/>
         <v>146.39595219199003</v>
       </c>
-      <c r="O41" s="56">
+      <c r="O41" s="55">
         <f t="shared" si="17"/>
         <v>0.31117465260340577</v>
       </c>
@@ -8444,23 +8486,23 @@
       </c>
     </row>
     <row r="48" spans="1:18" ht="18" x14ac:dyDescent="0.3">
-      <c r="A48" s="51">
+      <c r="A48" s="50">
         <f t="shared" ref="A48:A57" si="18">K17*1500/H17</f>
         <v>15.815560228296786</v>
       </c>
-      <c r="B48" s="52">
+      <c r="B48" s="51">
         <f>L17*1500/H17</f>
         <v>2.7150694945412757</v>
       </c>
-      <c r="C48" s="51">
+      <c r="C48" s="50">
         <f>M17*1500/H17</f>
         <v>115.20985252536632</v>
       </c>
-      <c r="D48" s="51">
+      <c r="D48" s="50">
         <f>N17*1500/H17</f>
         <v>316.69012611752606</v>
       </c>
-      <c r="E48" s="56">
+      <c r="E48" s="55">
         <f>C48/D48</f>
         <v>0.36379363618874266</v>
       </c>
@@ -8483,23 +8525,23 @@
       </c>
     </row>
     <row r="49" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A49" s="51">
+      <c r="A49" s="50">
         <f t="shared" si="18"/>
         <v>14.178544636159041</v>
       </c>
-      <c r="B49" s="52">
+      <c r="B49" s="51">
         <f t="shared" ref="B49:B57" si="19">L18*1500/H18</f>
         <v>3.6640096380168408</v>
       </c>
-      <c r="C49" s="51">
+      <c r="C49" s="50">
         <f t="shared" ref="C49:C57" si="20">M18*1500/H18</f>
         <v>139.53036014849988</v>
       </c>
-      <c r="D49" s="51">
+      <c r="D49" s="50">
         <f t="shared" ref="D49:D57" si="21">N18*1500/H18</f>
         <v>316.27561024564432</v>
       </c>
-      <c r="E49" s="56">
+      <c r="E49" s="55">
         <f t="shared" ref="E49:E57" si="22">C49/D49</f>
         <v>0.44116699368670798</v>
       </c>
@@ -8511,23 +8553,23 @@
       <c r="K49" s="9"/>
     </row>
     <row r="50" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A50" s="51">
+      <c r="A50" s="50">
         <f t="shared" si="18"/>
         <v>13.150007492881763</v>
       </c>
-      <c r="B50" s="52">
+      <c r="B50" s="51">
         <f t="shared" si="19"/>
         <v>4.073127891461227</v>
       </c>
-      <c r="C50" s="51">
+      <c r="C50" s="50">
         <f t="shared" si="20"/>
         <v>144.03083255501494</v>
       </c>
-      <c r="D50" s="51">
+      <c r="D50" s="50">
         <f t="shared" si="21"/>
         <v>311.71593565494709</v>
       </c>
-      <c r="E50" s="56">
+      <c r="E50" s="55">
         <f t="shared" si="22"/>
         <v>0.4620579703517288</v>
       </c>
@@ -8536,41 +8578,41 @@
       <c r="H50" s="11">
         <v>0</v>
       </c>
-      <c r="I50" s="52">
+      <c r="I50" s="51">
         <f t="shared" ref="I50:I57" si="23">(H50/3600)/(π*PumphjulsDiam*PumphjulsÖppning)</f>
         <v>0</v>
       </c>
-      <c r="J50" s="52">
+      <c r="J50" s="51">
         <f t="shared" ref="J50:J57" si="24">Euler_u2-(I50/TAN(RADIANS(Skovelvinkel)))</f>
         <v>8.6142470561432134</v>
       </c>
-      <c r="K50" s="51">
+      <c r="K50" s="50">
         <f t="shared" ref="K50:K57" si="25">Euler_u2*J50</f>
         <v>74.205252344272012</v>
       </c>
-      <c r="L50" s="53">
+      <c r="L50" s="52">
         <f t="shared" ref="L50:L57" si="26">K50/Tyngdacc</f>
         <v>7.5642459066536194</v>
       </c>
     </row>
     <row r="51" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A51" s="51">
+      <c r="A51" s="50">
         <f t="shared" si="18"/>
         <v>11.932584269662922</v>
       </c>
-      <c r="B51" s="52">
+      <c r="B51" s="51">
         <f t="shared" si="19"/>
         <v>4.4635026767417019</v>
       </c>
-      <c r="C51" s="51">
+      <c r="C51" s="50">
         <f t="shared" si="20"/>
         <v>143.26558549920227</v>
       </c>
-      <c r="D51" s="51">
+      <c r="D51" s="50">
         <f t="shared" si="21"/>
         <v>306.74174519236811</v>
       </c>
-      <c r="E51" s="56">
+      <c r="E51" s="55">
         <f t="shared" si="22"/>
         <v>0.46705604223955755</v>
       </c>
@@ -8578,41 +8620,41 @@
       <c r="H51" s="11">
         <v>2</v>
       </c>
-      <c r="I51" s="52">
+      <c r="I51" s="51">
         <f t="shared" si="23"/>
         <v>0.14174207136658207</v>
       </c>
-      <c r="J51" s="52">
+      <c r="J51" s="51">
         <f t="shared" si="24"/>
         <v>8.310280203170219</v>
       </c>
-      <c r="K51" s="51">
+      <c r="K51" s="50">
         <f t="shared" si="25"/>
         <v>71.586806775884284</v>
       </c>
-      <c r="L51" s="53">
+      <c r="L51" s="52">
         <f t="shared" si="26"/>
         <v>7.2973299465733215</v>
       </c>
     </row>
     <row r="52" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A52" s="51">
+      <c r="A52" s="50">
         <f t="shared" si="18"/>
         <v>9.5737533592117057</v>
       </c>
-      <c r="B52" s="52">
+      <c r="B52" s="51">
         <f t="shared" si="19"/>
         <v>5.1805966351479329</v>
       </c>
-      <c r="C52" s="51">
+      <c r="C52" s="50">
         <f t="shared" si="20"/>
         <v>133.87129254068583</v>
       </c>
-      <c r="D52" s="51">
+      <c r="D52" s="50">
         <f t="shared" si="21"/>
         <v>289.33207857334185</v>
       </c>
-      <c r="E52" s="56">
+      <c r="E52" s="55">
         <f t="shared" si="22"/>
         <v>0.46269080566796272</v>
       </c>
@@ -8621,41 +8663,41 @@
       <c r="H52" s="11">
         <v>4</v>
       </c>
-      <c r="I52" s="52">
+      <c r="I52" s="51">
         <f t="shared" si="23"/>
         <v>0.28348414273316414</v>
       </c>
-      <c r="J52" s="52">
+      <c r="J52" s="51">
         <f t="shared" si="24"/>
         <v>8.0063133501972228</v>
       </c>
-      <c r="K52" s="51">
+      <c r="K52" s="50">
         <f t="shared" si="25"/>
         <v>68.968361207496528</v>
       </c>
-      <c r="L52" s="53">
+      <c r="L52" s="52">
         <f t="shared" si="26"/>
         <v>7.03041398649302</v>
       </c>
     </row>
     <row r="53" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A53" s="51">
+      <c r="A53" s="50">
         <f t="shared" si="18"/>
         <v>8.1337399583457319</v>
       </c>
-      <c r="B53" s="52">
+      <c r="B53" s="51">
         <f t="shared" si="19"/>
         <v>5.5676926564052183</v>
       </c>
-      <c r="C53" s="51">
+      <c r="C53" s="50">
         <f t="shared" si="20"/>
         <v>122.67168894541888</v>
       </c>
-      <c r="D53" s="51">
+      <c r="D53" s="50">
         <f t="shared" si="21"/>
         <v>274.82402305748656</v>
       </c>
-      <c r="E53" s="56">
+      <c r="E53" s="55">
         <f t="shared" si="22"/>
         <v>0.44636450474985923</v>
       </c>
@@ -8664,41 +8706,41 @@
       <c r="H53" s="11">
         <v>6</v>
       </c>
-      <c r="I53" s="52">
+      <c r="I53" s="51">
         <f t="shared" si="23"/>
         <v>0.42522621409974626</v>
       </c>
-      <c r="J53" s="52">
+      <c r="J53" s="51">
         <f t="shared" si="24"/>
         <v>7.7023464972242284</v>
       </c>
-      <c r="K53" s="51">
+      <c r="K53" s="50">
         <f t="shared" si="25"/>
         <v>66.349915639108801</v>
       </c>
-      <c r="L53" s="53">
+      <c r="L53" s="52">
         <f t="shared" si="26"/>
         <v>6.7634980264127211</v>
       </c>
     </row>
     <row r="54" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A54" s="51">
+      <c r="A54" s="50">
         <f t="shared" si="18"/>
         <v>7.2171072171072179</v>
       </c>
-      <c r="B54" s="52">
+      <c r="B54" s="51">
         <f t="shared" si="19"/>
         <v>5.7108608817935247</v>
       </c>
-      <c r="C54" s="51">
+      <c r="C54" s="50">
         <f t="shared" si="20"/>
         <v>111.84540573788756</v>
       </c>
-      <c r="D54" s="51">
+      <c r="D54" s="50">
         <f t="shared" si="21"/>
         <v>265.29015800421024</v>
       </c>
-      <c r="E54" s="56">
+      <c r="E54" s="55">
         <f t="shared" si="22"/>
         <v>0.42159651371654933</v>
       </c>
@@ -8707,41 +8749,41 @@
       <c r="H54" s="11">
         <v>8</v>
       </c>
-      <c r="I54" s="52">
+      <c r="I54" s="51">
         <f t="shared" si="23"/>
         <v>0.56696828546632827</v>
       </c>
-      <c r="J54" s="52">
+      <c r="J54" s="51">
         <f t="shared" si="24"/>
         <v>7.3983796442512331</v>
       </c>
-      <c r="K54" s="51">
+      <c r="K54" s="50">
         <f t="shared" si="25"/>
         <v>63.731470070721059</v>
       </c>
-      <c r="L54" s="53">
+      <c r="L54" s="52">
         <f t="shared" si="26"/>
         <v>6.4965820663324214</v>
       </c>
     </row>
     <row r="55" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A55" s="51">
+      <c r="A55" s="50">
         <f t="shared" si="18"/>
         <v>6.403794841387489</v>
       </c>
-      <c r="B55" s="52">
+      <c r="B55" s="51">
         <f t="shared" si="19"/>
         <v>5.8498306030139506</v>
       </c>
-      <c r="C55" s="51">
+      <c r="C55" s="50">
         <f t="shared" si="20"/>
         <v>101.83740783427349</v>
       </c>
-      <c r="D55" s="51">
+      <c r="D55" s="50">
         <f t="shared" si="21"/>
         <v>256.1708088228155</v>
       </c>
-      <c r="E55" s="56">
+      <c r="E55" s="55">
         <f t="shared" si="22"/>
         <v>0.39753712884870857</v>
       </c>
@@ -8750,41 +8792,41 @@
       <c r="H55" s="11">
         <v>10</v>
       </c>
-      <c r="I55" s="52">
+      <c r="I55" s="51">
         <f t="shared" si="23"/>
         <v>0.70871035683291039</v>
       </c>
-      <c r="J55" s="52">
+      <c r="J55" s="51">
         <f t="shared" si="24"/>
         <v>7.0944127912782378</v>
       </c>
-      <c r="K55" s="51">
+      <c r="K55" s="50">
         <f t="shared" si="25"/>
         <v>61.113024502333317</v>
       </c>
-      <c r="L55" s="53">
+      <c r="L55" s="52">
         <f t="shared" si="26"/>
         <v>6.2296661062521217</v>
       </c>
     </row>
     <row r="56" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A56" s="51">
+      <c r="A56" s="50">
         <f t="shared" si="18"/>
         <v>5.4886162034299231</v>
       </c>
-      <c r="B56" s="52">
+      <c r="B56" s="51">
         <f t="shared" si="19"/>
         <v>5.973186981911609</v>
       </c>
-      <c r="C56" s="51">
+      <c r="C56" s="50">
         <f t="shared" si="20"/>
         <v>89.361998239595707</v>
       </c>
-      <c r="D56" s="51">
+      <c r="D56" s="50">
         <f t="shared" si="21"/>
         <v>244.56436441013128</v>
       </c>
-      <c r="E56" s="56">
+      <c r="E56" s="55">
         <f t="shared" si="22"/>
         <v>0.36539255608693993</v>
       </c>
@@ -8792,42 +8834,42 @@
       <c r="H56" s="11">
         <v>12</v>
       </c>
-      <c r="I56" s="52">
+      <c r="I56" s="51">
         <f t="shared" si="23"/>
         <v>0.85045242819949252</v>
       </c>
-      <c r="J56" s="52">
+      <c r="J56" s="51">
         <f t="shared" si="24"/>
         <v>6.7904459383052433</v>
       </c>
-      <c r="K56" s="51">
+      <c r="K56" s="50">
         <f t="shared" si="25"/>
         <v>58.494578933945583</v>
       </c>
-      <c r="L56" s="53">
+      <c r="L56" s="52">
         <f t="shared" si="26"/>
         <v>5.9627501461718229</v>
       </c>
       <c r="M56" s="19"/>
     </row>
     <row r="57" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A57" s="51">
+      <c r="A57" s="50">
         <f t="shared" si="18"/>
         <v>4.7759433962264151</v>
       </c>
-      <c r="B57" s="52">
+      <c r="B57" s="51">
         <f t="shared" si="19"/>
         <v>6.0003453692180724</v>
       </c>
-      <c r="C57" s="51">
+      <c r="C57" s="50">
         <f t="shared" si="20"/>
         <v>78.343245297999516</v>
       </c>
-      <c r="D57" s="51">
+      <c r="D57" s="50">
         <f t="shared" si="21"/>
         <v>232.12888825368395</v>
       </c>
-      <c r="E57" s="56">
+      <c r="E57" s="55">
         <f t="shared" si="22"/>
         <v>0.33749890367967239</v>
       </c>
@@ -8836,19 +8878,19 @@
       <c r="H57" s="11">
         <v>14</v>
       </c>
-      <c r="I57" s="52">
+      <c r="I57" s="51">
         <f t="shared" si="23"/>
         <v>0.99219449956607453</v>
       </c>
-      <c r="J57" s="52">
+      <c r="J57" s="51">
         <f t="shared" si="24"/>
         <v>6.4864790853322489</v>
       </c>
-      <c r="K57" s="51">
+      <c r="K57" s="50">
         <f t="shared" si="25"/>
         <v>55.876133365557848</v>
       </c>
-      <c r="L57" s="53">
+      <c r="L57" s="52">
         <f t="shared" si="26"/>
         <v>5.6958341860915231</v>
       </c>
@@ -8958,45 +9000,45 @@
       <c r="N62" s="9"/>
     </row>
     <row r="63" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A63" s="51">
+      <c r="A63" s="50">
         <f>K32*1200/H32</f>
         <v>12.534631224260577</v>
       </c>
-      <c r="B63" s="52">
+      <c r="B63" s="51">
         <f>L32*1200/H32</f>
         <v>1.9452054144732032</v>
       </c>
-      <c r="C63" s="51">
+      <c r="C63" s="50">
         <f>M32*1200/H32</f>
         <v>65.610179671330471</v>
       </c>
-      <c r="D63" s="51">
+      <c r="D63" s="50">
         <f>N32*1200/H32</f>
         <v>185.70311060294719</v>
       </c>
-      <c r="E63" s="56">
+      <c r="E63" s="55">
         <f>C63/D63</f>
         <v>0.35330684261725664</v>
       </c>
       <c r="F63" s="5"/>
       <c r="G63" s="24"/>
-      <c r="H63" s="51">
+      <c r="H63" s="50">
         <f>K32*1500/H32</f>
         <v>15.66828903032572</v>
       </c>
-      <c r="I63" s="52">
+      <c r="I63" s="51">
         <f>L32*1500/H32</f>
         <v>2.4315067680915039</v>
       </c>
-      <c r="J63" s="51">
+      <c r="J63" s="50">
         <f>M32*1500/H32</f>
         <v>82.012724589163071</v>
       </c>
-      <c r="K63" s="51">
+      <c r="K63" s="50">
         <f>N32*1500/H32</f>
         <v>232.12888825368404</v>
       </c>
-      <c r="L63" s="56">
+      <c r="L63" s="55">
         <f>J63/K63</f>
         <v>0.35330684261725653</v>
       </c>
@@ -9004,45 +9046,45 @@
       <c r="N63" s="30"/>
     </row>
     <row r="64" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A64" s="51">
+      <c r="A64" s="50">
         <f t="shared" ref="A64:A72" si="27">K33*1200/H33</f>
         <v>11.51084517576664</v>
       </c>
-      <c r="B64" s="52">
+      <c r="B64" s="51">
         <f t="shared" ref="B64:B72" si="28">L33*1200/H33</f>
         <v>2.2599733734672474</v>
       </c>
-      <c r="C64" s="51">
+      <c r="C64" s="50">
         <f t="shared" ref="C64:C72" si="29">M33*1200/H33</f>
         <v>70.07970191563588</v>
       </c>
-      <c r="D64" s="51">
+      <c r="D64" s="50">
         <f t="shared" ref="D64:D72" si="30">N33*1200/H33</f>
         <v>184.0450471154208</v>
       </c>
-      <c r="E64" s="56">
+      <c r="E64" s="55">
         <f t="shared" ref="E64:E72" si="31">C64/D64</f>
         <v>0.38077472343869462</v>
       </c>
       <c r="F64" s="5"/>
       <c r="G64" s="24"/>
-      <c r="H64" s="51">
+      <c r="H64" s="50">
         <f t="shared" ref="H64:H72" si="32">K33*1500/H33</f>
         <v>14.3885564697083</v>
       </c>
-      <c r="I64" s="52">
+      <c r="I64" s="51">
         <f t="shared" ref="I64:I72" si="33">L33*1500/H33</f>
         <v>2.8249667168340591</v>
       </c>
-      <c r="J64" s="51">
+      <c r="J64" s="50">
         <f t="shared" ref="J64:J72" si="34">M33*1500/H33</f>
         <v>87.599627394544854</v>
       </c>
-      <c r="K64" s="51">
+      <c r="K64" s="50">
         <f t="shared" ref="K64:K72" si="35">N33*1500/H33</f>
         <v>230.05630889427601</v>
       </c>
-      <c r="L64" s="56">
+      <c r="L64" s="55">
         <f t="shared" ref="L64:L72" si="36">J64/K64</f>
         <v>0.38077472343869462</v>
       </c>
@@ -9050,44 +9092,44 @@
       <c r="N64" s="30"/>
     </row>
     <row r="65" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A65" s="51">
+      <c r="A65" s="50">
         <f t="shared" si="27"/>
         <v>10.594170403587444</v>
       </c>
-      <c r="B65" s="52">
+      <c r="B65" s="51">
         <f t="shared" si="28"/>
         <v>2.5946186722645717</v>
       </c>
-      <c r="C65" s="51">
+      <c r="C65" s="50">
         <f t="shared" si="29"/>
         <v>74.104897412001762</v>
       </c>
-      <c r="D65" s="51">
+      <c r="D65" s="50">
         <f t="shared" si="30"/>
         <v>180.72892014036827</v>
       </c>
-      <c r="E65" s="56">
+      <c r="E65" s="55">
         <f t="shared" si="31"/>
         <v>0.41003342107309709</v>
       </c>
       <c r="F65" s="5"/>
-      <c r="H65" s="51">
+      <c r="H65" s="50">
         <f t="shared" si="32"/>
         <v>13.242713004484306</v>
       </c>
-      <c r="I65" s="52">
+      <c r="I65" s="51">
         <f t="shared" si="33"/>
         <v>3.2432733403307146</v>
       </c>
-      <c r="J65" s="51">
+      <c r="J65" s="50">
         <f t="shared" si="34"/>
         <v>92.631121765002206</v>
       </c>
-      <c r="K65" s="51">
+      <c r="K65" s="50">
         <f t="shared" si="35"/>
         <v>225.91115017546034</v>
       </c>
-      <c r="L65" s="56">
+      <c r="L65" s="55">
         <f t="shared" si="36"/>
         <v>0.41003342107309709</v>
       </c>
@@ -9095,45 +9137,45 @@
       <c r="N65" s="30"/>
     </row>
     <row r="66" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A66" s="51">
+      <c r="A66" s="50">
         <f t="shared" si="27"/>
         <v>9.6446511627906961</v>
       </c>
-      <c r="B66" s="52">
+      <c r="B66" s="51">
         <f t="shared" si="28"/>
         <v>2.9118264014121946</v>
       </c>
-      <c r="C66" s="51">
+      <c r="C66" s="50">
         <f t="shared" si="29"/>
         <v>76.03626657935331</v>
       </c>
-      <c r="D66" s="51">
+      <c r="D66" s="50">
         <f t="shared" si="30"/>
         <v>176.74956777030508</v>
       </c>
-      <c r="E66" s="56">
+      <c r="E66" s="55">
         <f t="shared" si="31"/>
         <v>0.43019209347185644</v>
       </c>
       <c r="F66" s="5"/>
       <c r="G66" s="24"/>
-      <c r="H66" s="51">
+      <c r="H66" s="50">
         <f t="shared" si="32"/>
         <v>12.055813953488371</v>
       </c>
-      <c r="I66" s="52">
+      <c r="I66" s="51">
         <f t="shared" si="33"/>
         <v>3.6397830017652431</v>
       </c>
-      <c r="J66" s="51">
+      <c r="J66" s="50">
         <f t="shared" si="34"/>
         <v>95.045333224191637</v>
       </c>
-      <c r="K66" s="51">
+      <c r="K66" s="50">
         <f t="shared" si="35"/>
         <v>220.93695971288133</v>
       </c>
-      <c r="L66" s="56">
+      <c r="L66" s="55">
         <f t="shared" si="36"/>
         <v>0.4301920934718565</v>
       </c>
@@ -9141,45 +9183,45 @@
       <c r="N66" s="30"/>
     </row>
     <row r="67" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A67" s="51">
+      <c r="A67" s="50">
         <f t="shared" si="27"/>
         <v>8.7502328180294278</v>
       </c>
-      <c r="B67" s="52">
+      <c r="B67" s="51">
         <f t="shared" si="28"/>
         <v>3.1549971800717365</v>
       </c>
-      <c r="C67" s="51">
+      <c r="C67" s="50">
         <f t="shared" si="29"/>
         <v>74.662460874386881</v>
       </c>
-      <c r="D67" s="51">
+      <c r="D67" s="50">
         <f t="shared" si="30"/>
         <v>174.09666619026299</v>
       </c>
-      <c r="E67" s="56">
+      <c r="E67" s="55">
         <f t="shared" si="31"/>
         <v>0.42885635037256481</v>
       </c>
       <c r="F67" s="5"/>
       <c r="G67" s="24"/>
-      <c r="H67" s="51">
+      <c r="H67" s="50">
         <f t="shared" si="32"/>
         <v>10.937791022536784</v>
       </c>
-      <c r="I67" s="52">
+      <c r="I67" s="51">
         <f t="shared" si="33"/>
         <v>3.9437464750896702</v>
       </c>
-      <c r="J67" s="51">
+      <c r="J67" s="50">
         <f t="shared" si="34"/>
         <v>93.328076092983594</v>
       </c>
-      <c r="K67" s="51">
+      <c r="K67" s="50">
         <f t="shared" si="35"/>
         <v>217.62083273782875</v>
       </c>
-      <c r="L67" s="56">
+      <c r="L67" s="55">
         <f t="shared" si="36"/>
         <v>0.42885635037256475</v>
       </c>
@@ -9187,45 +9229,45 @@
       <c r="N67" s="30"/>
     </row>
     <row r="68" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A68" s="51">
+      <c r="A68" s="50">
         <f t="shared" si="27"/>
         <v>7.9396984924623117</v>
       </c>
-      <c r="B68" s="52">
+      <c r="B68" s="51">
         <f t="shared" si="28"/>
         <v>3.3072547467102695</v>
       </c>
-      <c r="C68" s="51">
+      <c r="C68" s="50">
         <f t="shared" si="29"/>
         <v>71.068772091997673</v>
       </c>
-      <c r="D68" s="51">
+      <c r="D68" s="50">
         <f t="shared" si="30"/>
         <v>169.12247572768405</v>
       </c>
-      <c r="E68" s="56">
+      <c r="E68" s="55">
         <f t="shared" si="31"/>
         <v>0.42022074112982172</v>
       </c>
       <c r="F68" s="5"/>
       <c r="G68" s="24"/>
-      <c r="H68" s="51">
+      <c r="H68" s="50">
         <f t="shared" si="32"/>
         <v>9.924623115577889</v>
       </c>
-      <c r="I68" s="52">
+      <c r="I68" s="51">
         <f t="shared" si="33"/>
         <v>4.1340684333878368</v>
       </c>
-      <c r="J68" s="51">
+      <c r="J68" s="50">
         <f t="shared" si="34"/>
         <v>88.835965114997094</v>
       </c>
-      <c r="K68" s="51">
+      <c r="K68" s="50">
         <f t="shared" si="35"/>
         <v>211.40309465960505</v>
       </c>
-      <c r="L68" s="56">
+      <c r="L68" s="55">
         <f t="shared" si="36"/>
         <v>0.42022074112982177</v>
       </c>
@@ -9233,44 +9275,44 @@
       <c r="N68" s="30"/>
     </row>
     <row r="69" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A69" s="51">
+      <c r="A69" s="50">
         <f t="shared" si="27"/>
         <v>7.0208023774145607</v>
       </c>
-      <c r="B69" s="52">
+      <c r="B69" s="51">
         <f t="shared" si="28"/>
         <v>3.4544938078676126</v>
       </c>
-      <c r="C69" s="51">
+      <c r="C69" s="50">
         <f t="shared" si="29"/>
         <v>65.775859340181583</v>
       </c>
-      <c r="D69" s="51">
+      <c r="D69" s="50">
         <f t="shared" si="30"/>
         <v>165.80634875263141</v>
       </c>
-      <c r="E69" s="56">
+      <c r="E69" s="55">
         <f t="shared" si="31"/>
         <v>0.39670289970810119</v>
       </c>
       <c r="F69" s="5"/>
-      <c r="H69" s="51">
+      <c r="H69" s="50">
         <f t="shared" si="32"/>
         <v>8.776002971768202</v>
       </c>
-      <c r="I69" s="52">
+      <c r="I69" s="51">
         <f t="shared" si="33"/>
         <v>4.3181172598345157</v>
       </c>
-      <c r="J69" s="51">
+      <c r="J69" s="50">
         <f t="shared" si="34"/>
         <v>82.219824175226975</v>
       </c>
-      <c r="K69" s="51">
+      <c r="K69" s="50">
         <f t="shared" si="35"/>
         <v>207.25793594078925</v>
       </c>
-      <c r="L69" s="56">
+      <c r="L69" s="55">
         <f t="shared" si="36"/>
         <v>0.39670289970810119</v>
       </c>
@@ -9278,45 +9320,45 @@
       <c r="N69" s="30"/>
     </row>
     <row r="70" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A70" s="51">
+      <c r="A70" s="50">
         <f t="shared" si="27"/>
         <v>6.2068965517241379</v>
       </c>
-      <c r="B70" s="52">
+      <c r="B70" s="51">
         <f t="shared" si="28"/>
         <v>3.608242001526845</v>
       </c>
-      <c r="C70" s="51">
+      <c r="C70" s="50">
         <f t="shared" si="29"/>
         <v>60.851518368287621</v>
       </c>
-      <c r="D70" s="51">
+      <c r="D70" s="50">
         <f t="shared" si="30"/>
         <v>160.16893289504193</v>
       </c>
-      <c r="E70" s="56">
+      <c r="E70" s="55">
         <f t="shared" si="31"/>
         <v>0.37992085773689571</v>
       </c>
       <c r="F70" s="5"/>
       <c r="G70" s="24"/>
-      <c r="H70" s="51">
+      <c r="H70" s="50">
         <f t="shared" si="32"/>
         <v>7.7586206896551717</v>
       </c>
-      <c r="I70" s="52">
+      <c r="I70" s="51">
         <f t="shared" si="33"/>
         <v>4.5103025019085559</v>
       </c>
-      <c r="J70" s="51">
+      <c r="J70" s="50">
         <f t="shared" si="34"/>
         <v>76.064397960359514</v>
       </c>
-      <c r="K70" s="51">
+      <c r="K70" s="50">
         <f t="shared" si="35"/>
         <v>200.21116611880242</v>
       </c>
-      <c r="L70" s="56">
+      <c r="L70" s="55">
         <f t="shared" si="36"/>
         <v>0.37992085773689566</v>
       </c>
@@ -9324,45 +9366,45 @@
       <c r="N70" s="30"/>
     </row>
     <row r="71" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A71" s="51">
+      <c r="A71" s="50">
         <f t="shared" si="27"/>
         <v>5.3960029607697999</v>
       </c>
-      <c r="B71" s="52">
+      <c r="B71" s="51">
         <f t="shared" si="28"/>
         <v>3.662264016774023</v>
       </c>
-      <c r="C71" s="51">
+      <c r="C71" s="50">
         <f t="shared" si="29"/>
         <v>53.793212619817453</v>
       </c>
-      <c r="D71" s="51">
+      <c r="D71" s="50">
         <f t="shared" si="30"/>
         <v>152.87345354992615</v>
       </c>
-      <c r="E71" s="56">
+      <c r="E71" s="55">
         <f t="shared" si="31"/>
         <v>0.35188066580996946</v>
       </c>
       <c r="F71" s="5"/>
       <c r="G71" s="24"/>
-      <c r="H71" s="51">
+      <c r="H71" s="50">
         <f t="shared" si="32"/>
         <v>6.7450037009622505</v>
       </c>
-      <c r="I71" s="52">
+      <c r="I71" s="51">
         <f t="shared" si="33"/>
         <v>4.5778300209675287</v>
       </c>
-      <c r="J71" s="51">
+      <c r="J71" s="50">
         <f t="shared" si="34"/>
         <v>67.241515774771813</v>
       </c>
-      <c r="K71" s="51">
+      <c r="K71" s="50">
         <f t="shared" si="35"/>
         <v>191.09181693740771</v>
       </c>
-      <c r="L71" s="56">
+      <c r="L71" s="55">
         <f t="shared" si="36"/>
         <v>0.35188066580996941</v>
       </c>
@@ -9370,45 +9412,45 @@
       <c r="N71" s="30"/>
     </row>
     <row r="72" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A72" s="51">
+      <c r="A72" s="50">
         <f t="shared" si="27"/>
         <v>4.3853820598006648</v>
       </c>
-      <c r="B72" s="52">
+      <c r="B72" s="51">
         <f t="shared" si="28"/>
         <v>3.7935978686435008</v>
       </c>
-      <c r="C72" s="51">
+      <c r="C72" s="50">
         <f t="shared" si="29"/>
         <v>45.403365015834524</v>
       </c>
-      <c r="D72" s="51">
+      <c r="D72" s="50">
         <f t="shared" si="30"/>
         <v>145.90958690231565</v>
       </c>
-      <c r="E72" s="56">
+      <c r="E72" s="55">
         <f t="shared" si="31"/>
         <v>0.31117465260340582</v>
       </c>
       <c r="F72" s="5"/>
       <c r="G72" s="24"/>
-      <c r="H72" s="51">
+      <c r="H72" s="50">
         <f t="shared" si="32"/>
         <v>5.4817275747508312</v>
       </c>
-      <c r="I72" s="52">
+      <c r="I72" s="51">
         <f t="shared" si="33"/>
         <v>4.7419973358043759</v>
       </c>
-      <c r="J72" s="51">
+      <c r="J72" s="50">
         <f t="shared" si="34"/>
         <v>56.754206269793151</v>
       </c>
-      <c r="K72" s="51">
+      <c r="K72" s="50">
         <f t="shared" si="35"/>
         <v>182.38698362789458</v>
       </c>
-      <c r="L72" s="56">
+      <c r="L72" s="55">
         <f t="shared" si="36"/>
         <v>0.31117465260340577</v>
       </c>
@@ -9493,7 +9535,10 @@
       <c r="G78" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="H78" s="7"/>
+      <c r="H78" s="7">
+        <f>0.5+(2*0.3)+(2*1.1)</f>
+        <v>3.3000000000000003</v>
+      </c>
       <c r="I78" s="33" t="s">
         <v>30</v>
       </c>
@@ -9521,7 +9566,10 @@
       <c r="G79" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="H79" s="7"/>
+      <c r="H79" s="7">
+        <f>0.5+2+(3*0.3)+1.1+1.05</f>
+        <v>5.55</v>
+      </c>
       <c r="I79" s="35" t="s">
         <v>30</v>
       </c>
@@ -9605,6 +9653,9 @@
       <c r="G83" s="9"/>
       <c r="H83" s="9"/>
       <c r="I83" s="9"/>
+      <c r="L83" s="3" t="s">
+        <v>117</v>
+      </c>
       <c r="O83" s="5"/>
     </row>
     <row r="84" spans="1:15" x14ac:dyDescent="0.3">
@@ -9612,20 +9663,42 @@
         <v>0.01</v>
       </c>
       <c r="B84" s="36">
-        <f>4*Densitet*A84/3600/PI()/RörDiam_sug/Dynamisk_viskositet</f>
+        <f>(Densitet*((A84/3600)/(((RörDiam_sug/2)^2)*π))*RörDiam_sug)/Dynamisk_viskositet</f>
         <v>58.547434750075531</v>
       </c>
       <c r="C84" s="36">
-        <f>4*Densitet*A84/3600/PI()/RörDiam_tryck/Dynamisk_viskositet</f>
-        <v>70.256921700090615</v>
-      </c>
-      <c r="D84" s="17"/>
-      <c r="E84" s="17"/>
-      <c r="F84" s="17"/>
-      <c r="G84" s="17"/>
-      <c r="H84" s="17"/>
-      <c r="I84" s="17"/>
+        <f>(Densitet*((A84/3600)/(((RörDiam_tryck/2)^2)*π))*RörDiam_tryck)/Dynamisk_viskositet</f>
+        <v>70.256921700090629</v>
+      </c>
+      <c r="D84" s="56">
+        <f>8*((8/B84)^12+((-2.457*LN((7/B84)^0.9+0.27*(Ytråhet/RörDiam_sug)))^16+(37530/B84)^16)^-1.5)^(1/12)</f>
+        <v>1.0931307284973306</v>
+      </c>
+      <c r="E84" s="56">
+        <f>8*((8/C84)^12+((-2.457*LN((7/C84)^0.9+0.27*(Ytråhet/RörDiam_sug)))^16+(37530/C84)^16)^-1.5)^(1/12)</f>
+        <v>0.9109422737477757</v>
+      </c>
+      <c r="F84" s="59">
+        <f>D84*(RörLängd_sug/RörDiam_sug)*(((A84/3600)/(((RörDiam_sug/2)^2)*π))^2)/(2*Tyngdacc)</f>
+        <v>4.481280076578404E-6</v>
+      </c>
+      <c r="G84" s="58">
+        <f>E84*(RörLängd_tryck/RörDiam_tryck)*(((A84/3600)/(((RörDiam_tryck/2)^2)*π))^2)/(2*Tyngdacc)</f>
+        <v>3.7169529467171911E-5</v>
+      </c>
+      <c r="H84" s="58">
+        <f>H_stat+F84+G84+Engångs_sug*(((A84/3600)/(((RörDiam_sug/2)^2)*π))^2)/(2*Tyngdacc)+Engångs_tryck*(((A84/3600)/(((RörDiam_tryck/2)^2)*π))^2)/(2*Tyngdacc)</f>
+        <v>2.0000423792963899</v>
+      </c>
+      <c r="I84" s="59">
+        <f>($H$94/$A$94^2)*A84^2</f>
+        <v>3.8580104312922285E-6</v>
+      </c>
       <c r="K84" s="37"/>
+      <c r="L84" s="3">
+        <f>IF(C84&lt;2300, 64/C84, 0.25/(LOG10(((Ytråhet/RörDiam_tryck)/3.7)+(5.74/C84^0.9)))^2)</f>
+        <v>0.9109422737477757</v>
+      </c>
       <c r="O84" s="5"/>
     </row>
     <row r="85" spans="1:15" x14ac:dyDescent="0.3">
@@ -9633,19 +9706,37 @@
         <v>1</v>
       </c>
       <c r="B85" s="36">
-        <f>4*Densitet*A85/3600/PI()/RörDiam_sug/Dynamisk_viskositet</f>
-        <v>5854.7434750075518</v>
+        <f>(Densitet*((A85/3600)/(((RörDiam_sug/2)^2)*π))*RörDiam_sug)/Dynamisk_viskositet</f>
+        <v>5854.7434750075527</v>
       </c>
       <c r="C85" s="36">
-        <f>4*Densitet*A85/3600/PI()/RörDiam_tryck/Dynamisk_viskositet</f>
-        <v>7025.6921700090625</v>
-      </c>
-      <c r="D85" s="17"/>
-      <c r="E85" s="17"/>
-      <c r="F85" s="17"/>
-      <c r="G85" s="17"/>
-      <c r="H85" s="17"/>
-      <c r="I85" s="17"/>
+        <f>(Densitet*((A85/3600)/(((RörDiam_tryck/2)^2)*π))*RörDiam_tryck)/Dynamisk_viskositet</f>
+        <v>7025.6921700090634</v>
+      </c>
+      <c r="D85" s="56">
+        <f>8*((8/B85)^12+((-2.457*LN((7/B85)^0.9+0.27*(Ytråhet/RörDiam_sug)))^16+(37530/B85)^16)^-1.5)^(1/12)</f>
+        <v>3.8321925128009915E-2</v>
+      </c>
+      <c r="E85" s="56">
+        <f>8*((8/C85)^12+((-2.457*LN((7/C85)^0.9+0.27*(Ytråhet/RörDiam_sug)))^16+(37530/C85)^16)^-1.5)^(1/12)</f>
+        <v>3.6611859393007894E-2</v>
+      </c>
+      <c r="F85" s="57">
+        <f>D85*(RörLängd_sug/RörDiam_sug)*(((A85/3600)/(((RörDiam_sug/2)^2)*π))^2)/(2*Tyngdacc)</f>
+        <v>1.5710040445789141E-3</v>
+      </c>
+      <c r="G85" s="56">
+        <f>E85*(RörLängd_tryck/RörDiam_tryck)*(((A85/3600)/(((RörDiam_tryck/2)^2)*π))^2)/(2*Tyngdacc)</f>
+        <v>1.4938878409469404E-2</v>
+      </c>
+      <c r="H85" s="51">
+        <f>H_stat+F85+G85+Engångs_sug*(((A85/3600)/(((RörDiam_sug/2)^2)*π))^2)/(2*Tyngdacc)+Engångs_tryck*(((A85/3600)/(((RörDiam_tryck/2)^2)*π))^2)/(2*Tyngdacc)</f>
+        <v>2.0237947509139773</v>
+      </c>
+      <c r="I85" s="56">
+        <f t="shared" ref="I85:I98" si="37">($H$94/$A$94^2)*A85^2</f>
+        <v>3.8580104312922282E-2</v>
+      </c>
       <c r="K85" s="37"/>
       <c r="O85" s="5"/>
     </row>
@@ -9653,14 +9744,38 @@
       <c r="A86" s="11">
         <v>2</v>
       </c>
-      <c r="B86" s="36"/>
-      <c r="C86" s="36"/>
-      <c r="D86" s="17"/>
-      <c r="E86" s="17"/>
-      <c r="F86" s="17"/>
-      <c r="G86" s="17"/>
-      <c r="H86" s="17"/>
-      <c r="I86" s="17"/>
+      <c r="B86" s="36">
+        <f>(Densitet*((A86/3600)/(((RörDiam_sug/2)^2)*π))*RörDiam_sug)/Dynamisk_viskositet</f>
+        <v>11709.486950015105</v>
+      </c>
+      <c r="C86" s="36">
+        <f>(Densitet*((A86/3600)/(((RörDiam_tryck/2)^2)*π))*RörDiam_tryck)/Dynamisk_viskositet</f>
+        <v>14051.384340018127</v>
+      </c>
+      <c r="D86" s="56">
+        <f>8*((8/B86)^12+((-2.457*LN((7/B86)^0.9+0.27*(Ytråhet/RörDiam_sug)))^16+(37530/B86)^16)^-1.5)^(1/12)</f>
+        <v>3.2620438582158094E-2</v>
+      </c>
+      <c r="E86" s="56">
+        <f>8*((8/C86)^12+((-2.457*LN((7/C86)^0.9+0.27*(Ytråhet/RörDiam_sug)))^16+(37530/C86)^16)^-1.5)^(1/12)</f>
+        <v>3.1444182088847902E-2</v>
+      </c>
+      <c r="F86" s="57">
+        <f>D86*(RörLängd_sug/RörDiam_sug)*(((A86/3600)/(((RörDiam_sug/2)^2)*π))^2)/(2*Tyngdacc)</f>
+        <v>5.3490883641491745E-3</v>
+      </c>
+      <c r="G86" s="56">
+        <f>E86*(RörLängd_tryck/RörDiam_tryck)*(((A86/3600)/(((RörDiam_tryck/2)^2)*π))^2)/(2*Tyngdacc)</f>
+        <v>5.132116431106204E-2</v>
+      </c>
+      <c r="H86" s="51">
+        <f>H_stat+F86+G86+Engångs_sug*(((A86/3600)/(((RörDiam_sug/2)^2)*π))^2)/(2*Tyngdacc)+Engångs_tryck*(((A86/3600)/(((RörDiam_tryck/2)^2)*π))^2)/(2*Tyngdacc)</f>
+        <v>2.0858097265149258</v>
+      </c>
+      <c r="I86" s="56">
+        <f t="shared" si="37"/>
+        <v>0.15432041725168913</v>
+      </c>
       <c r="K86" s="37"/>
       <c r="O86" s="5"/>
     </row>
@@ -9668,14 +9783,38 @@
       <c r="A87" s="11">
         <v>3</v>
       </c>
-      <c r="B87" s="36"/>
-      <c r="C87" s="36"/>
-      <c r="D87" s="17"/>
-      <c r="E87" s="17"/>
-      <c r="F87" s="17"/>
-      <c r="G87" s="17"/>
-      <c r="H87" s="17"/>
-      <c r="I87" s="17"/>
+      <c r="B87" s="36">
+        <f>(Densitet*((A87/3600)/(((RörDiam_sug/2)^2)*π))*RörDiam_sug)/Dynamisk_viskositet</f>
+        <v>17564.230425022655</v>
+      </c>
+      <c r="C87" s="36">
+        <f>(Densitet*((A87/3600)/(((RörDiam_tryck/2)^2)*π))*RörDiam_tryck)/Dynamisk_viskositet</f>
+        <v>21077.076510027189</v>
+      </c>
+      <c r="D87" s="56">
+        <f>8*((8/B87)^12+((-2.457*LN((7/B87)^0.9+0.27*(Ytråhet/RörDiam_sug)))^16+(37530/B87)^16)^-1.5)^(1/12)</f>
+        <v>3.0158934944615735E-2</v>
+      </c>
+      <c r="E87" s="56">
+        <f>8*((8/C87)^12+((-2.457*LN((7/C87)^0.9+0.27*(Ytråhet/RörDiam_sug)))^16+(37530/C87)^16)^-1.5)^(1/12)</f>
+        <v>2.9224396022782723E-2</v>
+      </c>
+      <c r="F87" s="56">
+        <f>D87*(RörLängd_sug/RörDiam_sug)*(((A87/3600)/(((RörDiam_sug/2)^2)*π))^2)/(2*Tyngdacc)</f>
+        <v>1.1127266638595338E-2</v>
+      </c>
+      <c r="G87" s="56">
+        <f>E87*(RörLängd_tryck/RörDiam_tryck)*(((A87/3600)/(((RörDiam_tryck/2)^2)*π))^2)/(2*Tyngdacc)</f>
+        <v>0.10732088875336367</v>
+      </c>
+      <c r="H87" s="51">
+        <f>H_stat+F87+G87+Engångs_sug*(((A87/3600)/(((RörDiam_sug/2)^2)*π))^2)/(2*Tyngdacc)+Engångs_tryck*(((A87/3600)/(((RörDiam_tryck/2)^2)*π))^2)/(2*Tyngdacc)</f>
+        <v>2.1840119715313184</v>
+      </c>
+      <c r="I87" s="56">
+        <f t="shared" si="37"/>
+        <v>0.34722093881630056</v>
+      </c>
       <c r="K87" s="37"/>
       <c r="O87" s="5"/>
     </row>
@@ -9683,199 +9822,463 @@
       <c r="A88" s="11">
         <v>4</v>
       </c>
-      <c r="B88" s="36"/>
-      <c r="C88" s="36"/>
-      <c r="D88" s="17"/>
-      <c r="E88" s="17"/>
-      <c r="F88" s="17"/>
-      <c r="G88" s="17"/>
-      <c r="H88" s="17"/>
-      <c r="I88" s="17"/>
+      <c r="B88" s="36">
+        <f>(Densitet*((A88/3600)/(((RörDiam_sug/2)^2)*π))*RörDiam_sug)/Dynamisk_viskositet</f>
+        <v>23418.973900030211</v>
+      </c>
+      <c r="C88" s="36">
+        <f>(Densitet*((A88/3600)/(((RörDiam_tryck/2)^2)*π))*RörDiam_tryck)/Dynamisk_viskositet</f>
+        <v>28102.768680036253</v>
+      </c>
+      <c r="D88" s="56">
+        <f>8*((8/B88)^12+((-2.457*LN((7/B88)^0.9+0.27*(Ytråhet/RörDiam_sug)))^16+(37530/B88)^16)^-1.5)^(1/12)</f>
+        <v>2.8728264924052185E-2</v>
+      </c>
+      <c r="E88" s="56">
+        <f>8*((8/C88)^12+((-2.457*LN((7/C88)^0.9+0.27*(Ytråhet/RörDiam_sug)))^16+(37530/C88)^16)^-1.5)^(1/12)</f>
+        <v>2.794059197957208E-2</v>
+      </c>
+      <c r="F88" s="56">
+        <f>D88*(RörLängd_sug/RörDiam_sug)*(((A88/3600)/(((RörDiam_sug/2)^2)*π))^2)/(2*Tyngdacc)</f>
+        <v>1.8843404234484204E-2</v>
+      </c>
+      <c r="G88" s="56">
+        <f>E88*(RörLängd_tryck/RörDiam_tryck)*(((A88/3600)/(((RörDiam_tryck/2)^2)*π))^2)/(2*Tyngdacc)</f>
+        <v>0.18241132275347408</v>
+      </c>
+      <c r="H88" s="51">
+        <f>H_stat+F88+G88+Engångs_sug*(((A88/3600)/(((RörDiam_sug/2)^2)*π))^2)/(2*Tyngdacc)+Engångs_tryck*(((A88/3600)/(((RörDiam_tryck/2)^2)*π))^2)/(2*Tyngdacc)</f>
+        <v>2.317812622346819</v>
+      </c>
+      <c r="I88" s="56">
+        <f t="shared" si="37"/>
+        <v>0.61728166900675652</v>
+      </c>
       <c r="K88" s="37"/>
     </row>
     <row r="89" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A89" s="11">
         <v>5</v>
       </c>
-      <c r="B89" s="36"/>
-      <c r="C89" s="36"/>
-      <c r="D89" s="17"/>
-      <c r="E89" s="17"/>
-      <c r="F89" s="17"/>
-      <c r="G89" s="17"/>
-      <c r="H89" s="17"/>
-      <c r="I89" s="17"/>
+      <c r="B89" s="36">
+        <f>(Densitet*((A89/3600)/(((RörDiam_sug/2)^2)*π))*RörDiam_sug)/Dynamisk_viskositet</f>
+        <v>29273.717375037762</v>
+      </c>
+      <c r="C89" s="36">
+        <f>(Densitet*((A89/3600)/(((RörDiam_tryck/2)^2)*π))*RörDiam_tryck)/Dynamisk_viskositet</f>
+        <v>35128.460850045311</v>
+      </c>
+      <c r="D89" s="56">
+        <f>8*((8/B89)^12+((-2.457*LN((7/B89)^0.9+0.27*(Ytråhet/RörDiam_sug)))^16+(37530/B89)^16)^-1.5)^(1/12)</f>
+        <v>2.7775940661754841E-2</v>
+      </c>
+      <c r="E89" s="56">
+        <f>8*((8/C89)^12+((-2.457*LN((7/C89)^0.9+0.27*(Ytråhet/RörDiam_sug)))^16+(37530/C89)^16)^-1.5)^(1/12)</f>
+        <v>2.7089706830084295E-2</v>
+      </c>
+      <c r="F89" s="56">
+        <f>D89*(RörLängd_sug/RörDiam_sug)*(((A89/3600)/(((RörDiam_sug/2)^2)*π))^2)/(2*Tyngdacc)</f>
+        <v>2.8466807823354017E-2</v>
+      </c>
+      <c r="G89" s="56">
+        <f>E89*(RörLängd_tryck/RörDiam_tryck)*(((A89/3600)/(((RörDiam_tryck/2)^2)*π))^2)/(2*Tyngdacc)</f>
+        <v>0.27633794294540087</v>
+      </c>
+      <c r="H89" s="51">
+        <f>H_stat+F89+G89+Engångs_sug*(((A89/3600)/(((RörDiam_sug/2)^2)*π))^2)/(2*Tyngdacc)+Engångs_tryck*(((A89/3600)/(((RörDiam_tryck/2)^2)*π))^2)/(2*Tyngdacc)</f>
+        <v>2.4869264622669736</v>
+      </c>
+      <c r="I89" s="56">
+        <f t="shared" si="37"/>
+        <v>0.96450260782305708</v>
+      </c>
       <c r="K89" s="37"/>
     </row>
     <row r="90" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A90" s="11">
         <v>6</v>
       </c>
-      <c r="B90" s="36"/>
-      <c r="C90" s="36"/>
-      <c r="D90" s="17"/>
-      <c r="E90" s="17"/>
-      <c r="F90" s="17"/>
-      <c r="G90" s="17"/>
-      <c r="H90" s="17"/>
-      <c r="I90" s="17"/>
+      <c r="B90" s="36">
+        <f>(Densitet*((A90/3600)/(((RörDiam_sug/2)^2)*π))*RörDiam_sug)/Dynamisk_viskositet</f>
+        <v>35128.460850045311</v>
+      </c>
+      <c r="C90" s="36">
+        <f>(Densitet*((A90/3600)/(((RörDiam_tryck/2)^2)*π))*RörDiam_tryck)/Dynamisk_viskositet</f>
+        <v>42154.153020054378</v>
+      </c>
+      <c r="D90" s="56">
+        <f>8*((8/B90)^12+((-2.457*LN((7/B90)^0.9+0.27*(Ytråhet/RörDiam_sug)))^16+(37530/B90)^16)^-1.5)^(1/12)</f>
+        <v>2.7089706830084295E-2</v>
+      </c>
+      <c r="E90" s="56">
+        <f>8*((8/C90)^12+((-2.457*LN((7/C90)^0.9+0.27*(Ytråhet/RörDiam_sug)))^16+(37530/C90)^16)^-1.5)^(1/12)</f>
+        <v>2.6478837337398559E-2</v>
+      </c>
+      <c r="F90" s="56">
+        <f>D90*(RörLängd_sug/RörDiam_sug)*(((A90/3600)/(((RörDiam_sug/2)^2)*π))^2)/(2*Tyngdacc)</f>
+        <v>3.9979447764091576E-2</v>
+      </c>
+      <c r="G90" s="56">
+        <f>E90*(RörLängd_tryck/RörDiam_tryck)*(((A90/3600)/(((RörDiam_tryck/2)^2)*π))^2)/(2*Tyngdacc)</f>
+        <v>0.3889534420475288</v>
+      </c>
+      <c r="H90" s="51">
+        <f>H_stat+F90+G90+Engångs_sug*(((A90/3600)/(((RörDiam_sug/2)^2)*π))^2)/(2*Tyngdacc)+Engångs_tryck*(((A90/3600)/(((RörDiam_tryck/2)^2)*π))^2)/(2*Tyngdacc)</f>
+        <v>2.6911881543690566</v>
+      </c>
+      <c r="I90" s="51">
+        <f t="shared" si="37"/>
+        <v>1.3888837552652022</v>
+      </c>
       <c r="K90" s="37"/>
     </row>
     <row r="91" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A91" s="11">
         <v>7</v>
       </c>
-      <c r="B91" s="36"/>
-      <c r="C91" s="36"/>
-      <c r="D91" s="17"/>
-      <c r="E91" s="17"/>
-      <c r="F91" s="17"/>
-      <c r="G91" s="17"/>
-      <c r="H91" s="17"/>
-      <c r="I91" s="17"/>
+      <c r="B91" s="36">
+        <f>(Densitet*((A91/3600)/(((RörDiam_sug/2)^2)*π))*RörDiam_sug)/Dynamisk_viskositet</f>
+        <v>40983.204325052866</v>
+      </c>
+      <c r="C91" s="36">
+        <f>(Densitet*((A91/3600)/(((RörDiam_tryck/2)^2)*π))*RörDiam_tryck)/Dynamisk_viskositet</f>
+        <v>49179.845190063432</v>
+      </c>
+      <c r="D91" s="56">
+        <f>8*((8/B91)^12+((-2.457*LN((7/B91)^0.9+0.27*(Ytråhet/RörDiam_sug)))^16+(37530/B91)^16)^-1.5)^(1/12)</f>
+        <v>2.6568562047799192E-2</v>
+      </c>
+      <c r="E91" s="56">
+        <f>8*((8/C91)^12+((-2.457*LN((7/C91)^0.9+0.27*(Ytråhet/RörDiam_sug)))^16+(37530/C91)^16)^-1.5)^(1/12)</f>
+        <v>2.6016407424642111E-2</v>
+      </c>
+      <c r="F91" s="56">
+        <f>D91*(RörLängd_sug/RörDiam_sug)*(((A91/3600)/(((RörDiam_sug/2)^2)*π))^2)/(2*Tyngdacc)</f>
+        <v>5.3369620563667931E-2</v>
+      </c>
+      <c r="G91" s="56">
+        <f>E91*(RörLängd_tryck/RörDiam_tryck)*(((A91/3600)/(((RörDiam_tryck/2)^2)*π))^2)/(2*Tyngdacc)</f>
+        <v>0.52016318556239094</v>
+      </c>
+      <c r="H91" s="51">
+        <f>H_stat+F91+G91+Engångs_sug*(((A91/3600)/(((RörDiam_sug/2)^2)*π))^2)/(2*Tyngdacc)+Engångs_tryck*(((A91/3600)/(((RörDiam_tryck/2)^2)*π))^2)/(2*Tyngdacc)</f>
+        <v>2.9304913606625691</v>
+      </c>
+      <c r="I91" s="51">
+        <f t="shared" si="37"/>
+        <v>1.8904251113331918</v>
+      </c>
       <c r="K91" s="37"/>
     </row>
     <row r="92" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A92" s="11">
         <v>8</v>
       </c>
-      <c r="B92" s="36"/>
-      <c r="C92" s="36"/>
-      <c r="D92" s="17"/>
-      <c r="E92" s="17"/>
-      <c r="F92" s="17"/>
-      <c r="G92" s="17"/>
-      <c r="H92" s="17"/>
-      <c r="I92" s="17"/>
+      <c r="B92" s="36">
+        <f>(Densitet*((A92/3600)/(((RörDiam_sug/2)^2)*π))*RörDiam_sug)/Dynamisk_viskositet</f>
+        <v>46837.947800060421</v>
+      </c>
+      <c r="C92" s="36">
+        <f>(Densitet*((A92/3600)/(((RörDiam_tryck/2)^2)*π))*RörDiam_tryck)/Dynamisk_viskositet</f>
+        <v>56205.537360072507</v>
+      </c>
+      <c r="D92" s="56">
+        <f>8*((8/B92)^12+((-2.457*LN((7/B92)^0.9+0.27*(Ytråhet/RörDiam_sug)))^16+(37530/B92)^16)^-1.5)^(1/12)</f>
+        <v>2.6157666398074673E-2</v>
+      </c>
+      <c r="E92" s="56">
+        <f>8*((8/C92)^12+((-2.457*LN((7/C92)^0.9+0.27*(Ytråhet/RörDiam_sug)))^16+(37530/C92)^16)^-1.5)^(1/12)</f>
+        <v>2.5652817623557908E-2</v>
+      </c>
+      <c r="F92" s="56">
+        <f>D92*(RörLängd_sug/RörDiam_sug)*(((A92/3600)/(((RörDiam_sug/2)^2)*π))^2)/(2*Tyngdacc)</f>
+        <v>6.8629203061551403E-2</v>
+      </c>
+      <c r="G92" s="56">
+        <f>E92*(RörLängd_tryck/RörDiam_tryck)*(((A92/3600)/(((RörDiam_tryck/2)^2)*π))^2)/(2*Tyngdacc)</f>
+        <v>0.6699019689329424</v>
+      </c>
+      <c r="H92" s="51">
+        <f>H_stat+F92+G92+Engångs_sug*(((A92/3600)/(((RörDiam_sug/2)^2)*π))^2)/(2*Tyngdacc)+Engångs_tryck*(((A92/3600)/(((RörDiam_tryck/2)^2)*π))^2)/(2*Tyngdacc)</f>
+        <v>3.204762753429935</v>
+      </c>
+      <c r="I92" s="51">
+        <f t="shared" si="37"/>
+        <v>2.4691266760270261</v>
+      </c>
       <c r="K92" s="37"/>
     </row>
     <row r="93" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A93" s="11">
         <v>9</v>
       </c>
-      <c r="B93" s="36"/>
-      <c r="C93" s="36"/>
-      <c r="D93" s="17"/>
-      <c r="E93" s="17"/>
-      <c r="F93" s="17"/>
-      <c r="G93" s="17"/>
-      <c r="H93" s="17"/>
-      <c r="I93" s="17"/>
+      <c r="B93" s="36">
+        <f>(Densitet*((A93/3600)/(((RörDiam_sug/2)^2)*π))*RörDiam_sug)/Dynamisk_viskositet</f>
+        <v>52692.691275067969</v>
+      </c>
+      <c r="C93" s="36">
+        <f>(Densitet*((A93/3600)/(((RörDiam_tryck/2)^2)*π))*RörDiam_tryck)/Dynamisk_viskositet</f>
+        <v>63231.22953008156</v>
+      </c>
+      <c r="D93" s="56">
+        <f>8*((8/B93)^12+((-2.457*LN((7/B93)^0.9+0.27*(Ytråhet/RörDiam_sug)))^16+(37530/B93)^16)^-1.5)^(1/12)</f>
+        <v>2.5824424473964859E-2</v>
+      </c>
+      <c r="E93" s="56">
+        <f>8*((8/C93)^12+((-2.457*LN((7/C93)^0.9+0.27*(Ytråhet/RörDiam_sug)))^16+(37530/C93)^16)^-1.5)^(1/12)</f>
+        <v>2.5358659128890969E-2</v>
+      </c>
+      <c r="F93" s="56">
+        <f>D93*(RörLängd_sug/RörDiam_sug)*(((A93/3600)/(((RörDiam_sug/2)^2)*π))^2)/(2*Tyngdacc)</f>
+        <v>8.57522759653149E-2</v>
+      </c>
+      <c r="G93" s="56">
+        <f>E93*(RörLängd_tryck/RörDiam_tryck)*(((A93/3600)/(((RörDiam_tryck/2)^2)*π))^2)/(2*Tyngdacc)</f>
+        <v>0.83812252265746989</v>
+      </c>
+      <c r="H93" s="51">
+        <f>H_stat+F93+G93+Engångs_sug*(((A93/3600)/(((RörDiam_sug/2)^2)*π))^2)/(2*Tyngdacc)+Engångs_tryck*(((A93/3600)/(((RörDiam_tryck/2)^2)*π))^2)/(2*Tyngdacc)</f>
+        <v>3.5139491438770154</v>
+      </c>
+      <c r="I93" s="51">
+        <f t="shared" si="37"/>
+        <v>3.1249884493467048</v>
+      </c>
       <c r="K93" s="37"/>
     </row>
     <row r="94" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A94" s="38">
         <v>10</v>
       </c>
-      <c r="B94" s="36"/>
-      <c r="C94" s="36"/>
-      <c r="D94" s="17"/>
-      <c r="E94" s="17"/>
-      <c r="F94" s="17"/>
-      <c r="G94" s="17"/>
-      <c r="H94" s="39"/>
-      <c r="I94" s="17"/>
+      <c r="B94" s="36">
+        <f>(Densitet*((A94/3600)/(((RörDiam_sug/2)^2)*π))*RörDiam_sug)/Dynamisk_viskositet</f>
+        <v>58547.434750075525</v>
+      </c>
+      <c r="C94" s="36">
+        <f>(Densitet*((A94/3600)/(((RörDiam_tryck/2)^2)*π))*RörDiam_tryck)/Dynamisk_viskositet</f>
+        <v>70256.921700090621</v>
+      </c>
+      <c r="D94" s="56">
+        <f>8*((8/B94)^12+((-2.457*LN((7/B94)^0.9+0.27*(Ytråhet/RörDiam_sug)))^16+(37530/B94)^16)^-1.5)^(1/12)</f>
+        <v>2.5548135310566166E-2</v>
+      </c>
+      <c r="E94" s="56">
+        <f>8*((8/C94)^12+((-2.457*LN((7/C94)^0.9+0.27*(Ytråhet/RörDiam_sug)))^16+(37530/C94)^16)^-1.5)^(1/12)</f>
+        <v>2.5115298425681609E-2</v>
+      </c>
+      <c r="F94" s="56">
+        <f>D94*(RörLängd_sug/RörDiam_sug)*(((A94/3600)/(((RörDiam_sug/2)^2)*π))^2)/(2*Tyngdacc)</f>
+        <v>0.1047343623011591</v>
+      </c>
+      <c r="G94" s="51">
+        <f>E94*(RörLängd_tryck/RörDiam_tryck)*(((A94/3600)/(((RörDiam_tryck/2)^2)*π))^2)/(2*Tyngdacc)</f>
+        <v>1.0247892229981916</v>
+      </c>
+      <c r="H94" s="60">
+        <f>H_stat+F94+G94+Engångs_sug*(((A94/3600)/(((RörDiam_sug/2)^2)*π))^2)/(2*Tyngdacc)+Engångs_tryck*(((A94/3600)/(((RörDiam_tryck/2)^2)*π))^2)/(2*Tyngdacc)</f>
+        <v>3.8580104312922283</v>
+      </c>
+      <c r="I94" s="51">
+        <f t="shared" si="37"/>
+        <v>3.8580104312922283</v>
+      </c>
       <c r="K94" s="37"/>
     </row>
     <row r="95" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A95" s="11">
         <v>11</v>
       </c>
-      <c r="B95" s="36"/>
-      <c r="C95" s="36"/>
-      <c r="D95" s="17"/>
-      <c r="E95" s="17"/>
-      <c r="F95" s="17"/>
-      <c r="G95" s="17"/>
-      <c r="H95" s="17"/>
-      <c r="I95" s="17"/>
+      <c r="B95" s="36">
+        <f>(Densitet*((A95/3600)/(((RörDiam_sug/2)^2)*π))*RörDiam_sug)/Dynamisk_viskositet</f>
+        <v>64402.178225083073</v>
+      </c>
+      <c r="C95" s="36">
+        <f>(Densitet*((A95/3600)/(((RörDiam_tryck/2)^2)*π))*RörDiam_tryck)/Dynamisk_viskositet</f>
+        <v>77282.613870099696</v>
+      </c>
+      <c r="D95" s="56">
+        <f>8*((8/B95)^12+((-2.457*LN((7/B95)^0.9+0.27*(Ytråhet/RörDiam_sug)))^16+(37530/B95)^16)^-1.5)^(1/12)</f>
+        <v>2.5314967129198923E-2</v>
+      </c>
+      <c r="E95" s="56">
+        <f>8*((8/C95)^12+((-2.457*LN((7/C95)^0.9+0.27*(Ytråhet/RörDiam_sug)))^16+(37530/C95)^16)^-1.5)^(1/12)</f>
+        <v>2.4910312727500619E-2</v>
+      </c>
+      <c r="F95" s="56">
+        <f>D95*(RörLängd_sug/RörDiam_sug)*(((A95/3600)/(((RörDiam_sug/2)^2)*π))^2)/(2*Tyngdacc)</f>
+        <v>0.12557197451527682</v>
+      </c>
+      <c r="G95" s="51">
+        <f>E95*(RörLängd_tryck/RörDiam_tryck)*(((A95/3600)/(((RörDiam_tryck/2)^2)*π))^2)/(2*Tyngdacc)</f>
+        <v>1.2298743859738575</v>
+      </c>
+      <c r="H95" s="51">
+        <f>H_stat+F95+G95+Engångs_sug*(((A95/3600)/(((RörDiam_sug/2)^2)*π))^2)/(2*Tyngdacc)+Engångs_tryck*(((A95/3600)/(((RörDiam_tryck/2)^2)*π))^2)/(2*Tyngdacc)</f>
+        <v>4.2369154441405161</v>
+      </c>
+      <c r="I95" s="51">
+        <f t="shared" si="37"/>
+        <v>4.6681926218635965</v>
+      </c>
       <c r="K95" s="37"/>
     </row>
     <row r="96" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A96" s="11">
         <v>12</v>
       </c>
-      <c r="B96" s="36"/>
-      <c r="C96" s="36"/>
-      <c r="D96" s="17"/>
-      <c r="E96" s="17"/>
-      <c r="F96" s="17"/>
-      <c r="G96" s="17"/>
-      <c r="H96" s="17"/>
-      <c r="I96" s="17"/>
+      <c r="B96" s="36">
+        <f>(Densitet*((A96/3600)/(((RörDiam_sug/2)^2)*π))*RörDiam_sug)/Dynamisk_viskositet</f>
+        <v>70256.921700090621</v>
+      </c>
+      <c r="C96" s="36">
+        <f>(Densitet*((A96/3600)/(((RörDiam_tryck/2)^2)*π))*RörDiam_tryck)/Dynamisk_viskositet</f>
+        <v>84308.306040108757</v>
+      </c>
+      <c r="D96" s="56">
+        <f>8*((8/B96)^12+((-2.457*LN((7/B96)^0.9+0.27*(Ytråhet/RörDiam_sug)))^16+(37530/B96)^16)^-1.5)^(1/12)</f>
+        <v>2.5115298425681609E-2</v>
+      </c>
+      <c r="E96" s="56">
+        <f>8*((8/C96)^12+((-2.457*LN((7/C96)^0.9+0.27*(Ytråhet/RörDiam_sug)))^16+(37530/C96)^16)^-1.5)^(1/12)</f>
+        <v>2.4735078652284546E-2</v>
+      </c>
+      <c r="F96" s="56">
+        <f>D96*(RörLängd_sug/RörDiam_sug)*(((A96/3600)/(((RörDiam_sug/2)^2)*π))^2)/(2*Tyngdacc)</f>
+        <v>0.14826232971617359</v>
+      </c>
+      <c r="G96" s="51">
+        <f>E96*(RörLängd_tryck/RörDiam_tryck)*(((A96/3600)/(((RörDiam_tryck/2)^2)*π))^2)/(2*Tyngdacc)</f>
+        <v>1.453355954951099</v>
+      </c>
+      <c r="H96" s="51">
+        <f>H_stat+F96+G96+Engångs_sug*(((A96/3600)/(((RörDiam_sug/2)^2)*π))^2)/(2*Tyngdacc)+Engångs_tryck*(((A96/3600)/(((RörDiam_tryck/2)^2)*π))^2)/(2*Tyngdacc)</f>
+        <v>4.6506393428970156</v>
+      </c>
+      <c r="I96" s="51">
+        <f t="shared" si="37"/>
+        <v>5.555535021060809</v>
+      </c>
       <c r="K96" s="37"/>
     </row>
     <row r="97" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A97" s="11">
         <v>13</v>
       </c>
-      <c r="B97" s="36"/>
-      <c r="C97" s="36"/>
-      <c r="D97" s="17"/>
-      <c r="E97" s="17"/>
-      <c r="F97" s="17"/>
-      <c r="G97" s="17"/>
-      <c r="H97" s="17"/>
-      <c r="I97" s="17"/>
+      <c r="B97" s="36">
+        <f>(Densitet*((A97/3600)/(((RörDiam_sug/2)^2)*π))*RörDiam_sug)/Dynamisk_viskositet</f>
+        <v>76111.665175098169</v>
+      </c>
+      <c r="C97" s="36">
+        <f>(Densitet*((A97/3600)/(((RörDiam_tryck/2)^2)*π))*RörDiam_tryck)/Dynamisk_viskositet</f>
+        <v>91333.998210117803</v>
+      </c>
+      <c r="D97" s="56">
+        <f>8*((8/B97)^12+((-2.457*LN((7/B97)^0.9+0.27*(Ytråhet/RörDiam_sug)))^16+(37530/B97)^16)^-1.5)^(1/12)</f>
+        <v>2.4942213741927205E-2</v>
+      </c>
+      <c r="E97" s="56">
+        <f>8*((8/C97)^12+((-2.457*LN((7/C97)^0.9+0.27*(Ytråhet/RörDiam_sug)))^16+(37530/C97)^16)^-1.5)^(1/12)</f>
+        <v>2.4583410261233431E-2</v>
+      </c>
+      <c r="F97" s="56">
+        <f>D97*(RörLängd_sug/RörDiam_sug)*(((A97/3600)/(((RörDiam_sug/2)^2)*π))^2)/(2*Tyngdacc)</f>
+        <v>0.17280316249756403</v>
+      </c>
+      <c r="G97" s="51">
+        <f>E97*(RörLängd_tryck/RörDiam_tryck)*(((A97/3600)/(((RörDiam_tryck/2)^2)*π))^2)/(2*Tyngdacc)</f>
+        <v>1.695215990262547</v>
+      </c>
+      <c r="H97" s="51">
+        <f>H_stat+F97+G97+Engångs_sug*(((A97/3600)/(((RörDiam_sug/2)^2)*π))^2)/(2*Tyngdacc)+Engångs_tryck*(((A97/3600)/(((RörDiam_tryck/2)^2)*π))^2)/(2*Tyngdacc)</f>
+        <v>5.099161922488074</v>
+      </c>
+      <c r="I97" s="51">
+        <f t="shared" si="37"/>
+        <v>6.5200376288838653</v>
+      </c>
       <c r="K97" s="37"/>
     </row>
     <row r="98" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A98" s="11">
         <v>14</v>
       </c>
-      <c r="B98" s="36"/>
-      <c r="C98" s="36"/>
-      <c r="D98" s="17"/>
-      <c r="E98" s="17"/>
-      <c r="F98" s="17"/>
-      <c r="G98" s="17"/>
-      <c r="H98" s="17"/>
-      <c r="I98" s="17"/>
+      <c r="B98" s="36">
+        <f>(Densitet*((A98/3600)/(((RörDiam_sug/2)^2)*π))*RörDiam_sug)/Dynamisk_viskositet</f>
+        <v>81966.408650105732</v>
+      </c>
+      <c r="C98" s="36">
+        <f>(Densitet*((A98/3600)/(((RörDiam_tryck/2)^2)*π))*RörDiam_tryck)/Dynamisk_viskositet</f>
+        <v>98359.690380126864</v>
+      </c>
+      <c r="D98" s="56">
+        <f>8*((8/B98)^12+((-2.457*LN((7/B98)^0.9+0.27*(Ytråhet/RörDiam_sug)))^16+(37530/B98)^16)^-1.5)^(1/12)</f>
+        <v>2.4790605712953471E-2</v>
+      </c>
+      <c r="E98" s="56">
+        <f>8*((8/C98)^12+((-2.457*LN((7/C98)^0.9+0.27*(Ytråhet/RörDiam_sug)))^16+(37530/C98)^16)^-1.5)^(1/12)</f>
+        <v>2.4450747337404773E-2</v>
+      </c>
+      <c r="F98" s="56">
+        <f>D98*(RörLängd_sug/RörDiam_sug)*(((A98/3600)/(((RörDiam_sug/2)^2)*π))^2)/(2*Tyngdacc)</f>
+        <v>0.19919259733568023</v>
+      </c>
+      <c r="G98" s="51">
+        <f>E98*(RörLängd_tryck/RörDiam_tryck)*(((A98/3600)/(((RörDiam_tryck/2)^2)*π))^2)/(2*Tyngdacc)</f>
+        <v>1.9554396449617522</v>
+      </c>
+      <c r="H98" s="51">
+        <f>H_stat+F98+G98+Engångs_sug*(((A98/3600)/(((RörDiam_sug/2)^2)*π))^2)/(2*Tyngdacc)+Engångs_tryck*(((A98/3600)/(((RörDiam_tryck/2)^2)*π))^2)/(2*Tyngdacc)</f>
+        <v>5.5824664604434719</v>
+      </c>
+      <c r="I98" s="51">
+        <f t="shared" si="37"/>
+        <v>7.5617004453327672</v>
+      </c>
       <c r="K98" s="37"/>
     </row>
     <row r="105" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A105" s="40" t="s">
+      <c r="A105" s="39" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="106" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A106" s="41" t="s">
+      <c r="A106" s="40" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="107" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A107" s="42" t="s">
+      <c r="A107" s="41" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="126" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A126" s="40" t="s">
+      <c r="A126" s="39" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="127" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A127" s="41" t="s">
+      <c r="A127" s="40" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="128" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A128" s="42" t="s">
+      <c r="A128" s="41" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="144" s="3" customFormat="1" ht="69.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="145" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A145" s="43" t="s">
+      <c r="A145" s="42" t="s">
         <v>115</v>
       </c>
     </row>
     <row r="146" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A146" s="44" t="s">
+      <c r="A146" s="43" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="147" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A147" s="42"/>
+      <c r="A147" s="41"/>
     </row>
     <row r="150" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B150" s="9" t="s">
@@ -9901,24 +10304,24 @@
       <c r="A153" s="3">
         <v>1200</v>
       </c>
-      <c r="B153" s="45"/>
-      <c r="C153" s="46"/>
+      <c r="B153" s="44"/>
+      <c r="C153" s="45"/>
     </row>
     <row r="154" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A154" s="3">
         <v>1200</v>
       </c>
-      <c r="B154" s="45"/>
-      <c r="C154" s="46"/>
+      <c r="B154" s="44"/>
+      <c r="C154" s="45"/>
     </row>
     <row r="159" spans="1:3" ht="51.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="160" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A160" s="43" t="s">
+      <c r="A160" s="42" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="161" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A161" s="41" t="s">
+      <c r="A161" s="40" t="s">
         <v>45</v>
       </c>
     </row>
@@ -9942,9 +10345,9 @@
       <c r="A166" s="5" t="s">
         <v>101</v>
       </c>
-      <c r="B166" s="45"/>
-      <c r="C166" s="46"/>
-      <c r="D166" s="47"/>
+      <c r="B166" s="44"/>
+      <c r="C166" s="45"/>
+      <c r="D166" s="46"/>
       <c r="E166" s="9"/>
     </row>
     <row r="168" spans="1:5" x14ac:dyDescent="0.3">
@@ -9988,8 +10391,8 @@
       <c r="A171" s="9">
         <v>1200</v>
       </c>
-      <c r="B171" s="45"/>
-      <c r="C171" s="46"/>
+      <c r="B171" s="44"/>
+      <c r="C171" s="45"/>
       <c r="D171" s="17"/>
       <c r="E171" s="17"/>
     </row>
@@ -9997,8 +10400,8 @@
       <c r="A172" s="9">
         <v>1200</v>
       </c>
-      <c r="B172" s="45"/>
-      <c r="C172" s="46"/>
+      <c r="B172" s="44"/>
+      <c r="C172" s="45"/>
       <c r="D172" s="17"/>
       <c r="E172" s="17"/>
     </row>
@@ -10010,17 +10413,17 @@
     </row>
     <row r="175" spans="1:5" ht="59.25" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="176" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A176" s="43" t="s">
+      <c r="A176" s="42" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="177" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A177" s="41" t="s">
+      <c r="A177" s="40" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="178" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A178" s="42" t="s">
+      <c r="A178" s="41" t="s">
         <v>86</v>
       </c>
     </row>
@@ -10085,7 +10488,7 @@
       <c r="L180" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="M180" s="48">
+      <c r="M180" s="47">
         <v>0.8</v>
       </c>
     </row>
@@ -10117,7 +10520,7 @@
       <c r="L181" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="M181" s="48">
+      <c r="M181" s="47">
         <v>0.95</v>
       </c>
     </row>
@@ -10135,10 +10538,10 @@
       <c r="A183" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="C183" s="49"/>
-      <c r="D183" s="49"/>
-      <c r="E183" s="49"/>
-      <c r="F183" s="50"/>
+      <c r="C183" s="48"/>
+      <c r="D183" s="48"/>
+      <c r="E183" s="48"/>
+      <c r="F183" s="49"/>
       <c r="G183" s="17"/>
       <c r="H183" s="17"/>
       <c r="I183" s="17"/>
@@ -10148,10 +10551,10 @@
       <c r="A184" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="C184" s="49"/>
-      <c r="D184" s="49"/>
-      <c r="E184" s="49"/>
-      <c r="F184" s="50"/>
+      <c r="C184" s="48"/>
+      <c r="D184" s="48"/>
+      <c r="E184" s="48"/>
+      <c r="F184" s="49"/>
       <c r="G184" s="17"/>
       <c r="H184" s="17"/>
       <c r="I184" s="17"/>
@@ -10161,10 +10564,10 @@
       <c r="A185" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="C185" s="49"/>
-      <c r="D185" s="49"/>
-      <c r="E185" s="49"/>
-      <c r="F185" s="50"/>
+      <c r="C185" s="48"/>
+      <c r="D185" s="48"/>
+      <c r="E185" s="48"/>
+      <c r="F185" s="49"/>
       <c r="G185" s="17"/>
       <c r="H185" s="17"/>
       <c r="I185" s="17"/>
@@ -10174,10 +10577,10 @@
       <c r="A186" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="C186" s="49"/>
-      <c r="D186" s="49"/>
-      <c r="E186" s="49"/>
-      <c r="F186" s="50"/>
+      <c r="C186" s="48"/>
+      <c r="D186" s="48"/>
+      <c r="E186" s="48"/>
+      <c r="F186" s="49"/>
       <c r="G186" s="17"/>
       <c r="H186" s="17"/>
       <c r="I186" s="17"/>
@@ -10187,10 +10590,10 @@
       <c r="A187" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="C187" s="49"/>
-      <c r="D187" s="49"/>
-      <c r="E187" s="49"/>
-      <c r="F187" s="50"/>
+      <c r="C187" s="48"/>
+      <c r="D187" s="48"/>
+      <c r="E187" s="48"/>
+      <c r="F187" s="49"/>
       <c r="G187" s="17"/>
       <c r="H187" s="17"/>
       <c r="I187" s="17"/>

</xml_diff>